<commit_message>
feat: add Chinese frontier AI lab interviews
</commit_message>
<xml_diff>
--- a/data/scholar_tube_seed_list.xlsx
+++ b/data/scholar_tube_seed_list.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re63cdb0404ca4746"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="2" r:id="R9574f36bd140405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Areas" sheetId="3" r:id="R27414b4737744627"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Index" sheetId="4" r:id="Rc66aa74addac49ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="5" r:id="R7077e461c8d94a06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra2870e29109b4168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="2" r:id="R6f79ede3a94648df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Areas" sheetId="3" r:id="R0dee8fc2c53646ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Index" sheetId="4" r:id="R43f2a7cc892f4f87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="5" r:id="Rd68a06d8adb44dda"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -750,8 +750,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScholarTubeResources" displayName="ScholarTubeResources" ref="A1:T530" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:T530"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScholarTubeResources" displayName="ScholarTubeResources" ref="A1:T559" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:T559"/>
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Section"/>
@@ -1056,40 +1056,40 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="B2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="C2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="D2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="E2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="F2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="G2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="H2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="I2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="J2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="K2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="L2" s="30" t="str">
-        <x:v>Curated resources: 529 direct video links | Four priority areas: 354 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 558 direct video links | Four priority areas: 383 | YouTube + Bilibili, with Xiaohongshu fields reserved | Metadata checked: 2026-08-12</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
@@ -1120,23 +1120,23 @@
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" s="93" t="n">
-        <x:f>COUNTA('Resources'!$A$2:$A$530)</x:f>
-        <x:v>529</x:v>
+        <x:f>COUNTA('Resources'!$A$2:$A$559)</x:f>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="B5" s="94"/>
       <x:c r="D5" s="93" t="n">
-        <x:f>COUNTIF('Resources'!$B$2:$B$530,"Interview")</x:f>
-        <x:v>136</x:v>
+        <x:f>COUNTIF('Resources'!$B$2:$B$559,"Interview")</x:f>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="E5" s="94"/>
       <x:c r="G5" s="93" t="n">
-        <x:f>COUNTIF('Resources'!$B$2:$B$530,"Course")</x:f>
-        <x:v>198</x:v>
+        <x:f>COUNTIF('Resources'!$B$2:$B$559,"Course")</x:f>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="H5" s="94"/>
       <x:c r="J5" s="93" t="n">
-        <x:f>COUNTIF('Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>195</x:v>
+        <x:f>COUNTIF('Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="K5" s="94"/>
     </x:row>
@@ -1168,23 +1168,23 @@
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="93" t="n">
-        <x:f>COUNTIF('Resources'!$O$2:$O$530,"A | Official / Original Creator / Organizer")</x:f>
-        <x:v>323</x:v>
+        <x:f>COUNTIF('Resources'!$O$2:$O$559,"A | Official / Original Creator / Organizer")</x:f>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="B8" s="94"/>
       <x:c r="D8" s="93" t="n">
-        <x:f>COUNTIF('Resources'!$C$2:$C$530,"&lt;&gt;Other")</x:f>
-        <x:v>354</x:v>
+        <x:f>COUNTIF('Resources'!$C$2:$C$559,"&lt;&gt;Other")</x:f>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="E8" s="94"/>
       <x:c r="G8" s="93" t="n">
-        <x:f>COUNTIF('Resources'!$F$2:$F$530,"Chinese")</x:f>
-        <x:v>107</x:v>
+        <x:f>COUNTIF('Resources'!$F$2:$F$559,"Chinese")</x:f>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="H8" s="94"/>
       <x:c r="J8" s="93" t="n">
-        <x:f>COUNTIF('Resources'!$Q$2:$Q$530,"Verified")</x:f>
-        <x:v>529</x:v>
+        <x:f>COUNTIF('Resources'!$Q$2:$Q$559,"Verified")</x:f>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="K8" s="94"/>
     </x:row>
@@ -1260,100 +1260,100 @@
         <x:v>Robotics / Embodied AI</x:v>
       </x:c>
       <x:c r="B13" s="81" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A13)</x:f>
-        <x:v>67</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A13)</x:f>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C13" s="106" t="n">
         <x:f>B13/$A$5</x:f>
-        <x:v>0.1266540642722117</x:v>
+        <x:v>0.12365591397849462</x:v>
       </x:c>
       <x:c r="E13" s="34" t="str">
         <x:v>Stanford Online</x:v>
       </x:c>
       <x:c r="F13" s="76" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E13)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E13)</x:f>
         <x:v>44</x:v>
       </x:c>
       <x:c r="H13" s="34" t="str">
         <x:v>A | Official / Original Creator / Organizer</x:v>
       </x:c>
       <x:c r="I13" s="76" t="n">
-        <x:f>COUNTIF('Resources'!$O$2:$O$530,"A | Official / Original Creator / Organizer")</x:f>
-        <x:v>323</x:v>
+        <x:f>COUNTIF('Resources'!$O$2:$O$559,"A | Official / Original Creator / Organizer")</x:f>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="J13" s="34" t="str">
         <x:v>YouTube</x:v>
       </x:c>
       <x:c r="K13" s="76" t="n">
-        <x:f>COUNTIF('Resources'!$M$2:$M$530,"YouTube")</x:f>
+        <x:f>COUNTIF('Resources'!$M$2:$M$559,"YouTube")</x:f>
         <x:v>425</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="37" t="str">
-        <x:v>Robotics</x:v>
+        <x:v>Agents / Tool Use / Reasoning</x:v>
       </x:c>
       <x:c r="B14" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A14)</x:f>
-        <x:v>42</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A14)</x:f>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C14" s="107" t="n">
         <x:f>B14/$A$5</x:f>
-        <x:v>0.07939508506616257</x:v>
+        <x:v>0.11290322580645161</x:v>
       </x:c>
       <x:c r="E14" s="37" t="str">
         <x:v>Lex Fridman</x:v>
       </x:c>
       <x:c r="F14" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E14)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E14)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="H14" s="37" t="str">
         <x:v>B | University / Conference / Institution</x:v>
       </x:c>
       <x:c r="I14" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$O$2:$O$530,"B | University / Conference / Institution")</x:f>
-        <x:v>125</x:v>
+        <x:f>COUNTIF('Resources'!$O$2:$O$559,"B | University / Conference / Institution")</x:f>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="J14" s="37" t="str">
         <x:v>Bilibili</x:v>
       </x:c>
       <x:c r="K14" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$M$2:$M$530,"Bilibili")</x:f>
-        <x:v>104</x:v>
+        <x:f>COUNTIF('Resources'!$M$2:$M$559,"Bilibili")</x:f>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="37" t="str">
-        <x:v>Agents / Tool Use / Reasoning</x:v>
+        <x:v>Robotics</x:v>
       </x:c>
       <x:c r="B15" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A15)</x:f>
-        <x:v>41</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A15)</x:f>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C15" s="107" t="n">
         <x:f>B15/$A$5</x:f>
-        <x:v>0.07750472589792061</x:v>
+        <x:v>0.07526881720430108</x:v>
       </x:c>
       <x:c r="E15" s="37" t="str">
         <x:v>CMU Robotics Institute</x:v>
       </x:c>
       <x:c r="F15" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E15)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E15)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="H15" s="40" t="str">
         <x:v>C | Community Selection</x:v>
       </x:c>
       <x:c r="I15" s="80" t="n">
-        <x:f>COUNTIF('Resources'!$O$2:$O$530,"C | Community Selection")</x:f>
-        <x:v>81</x:v>
+        <x:f>COUNTIF('Resources'!$O$2:$O$559,"C | Community Selection")</x:f>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="J15" s="40" t="str">
         <x:v>Xiaohongshu</x:v>
       </x:c>
       <x:c r="K15" s="80" t="n">
-        <x:f>COUNTIF('Resources'!$M$2:$M$530,"Xiaohongshu")</x:f>
+        <x:f>COUNTIF('Resources'!$M$2:$M$559,"Xiaohongshu")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1362,18 +1362,18 @@
         <x:v>Agents</x:v>
       </x:c>
       <x:c r="B16" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A16)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A16)</x:f>
         <x:v>39</x:v>
       </x:c>
       <x:c r="C16" s="107" t="n">
         <x:f>B16/$A$5</x:f>
-        <x:v>0.07372400756143667</x:v>
+        <x:v>0.06989247311827956</x:v>
       </x:c>
       <x:c r="E16" s="37" t="str">
         <x:v>Dwarkesh Patel</x:v>
       </x:c>
       <x:c r="F16" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E16)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E16)</x:f>
         <x:v>9</x:v>
       </x:c>
     </x:row>
@@ -1382,73 +1382,73 @@
         <x:v>Vision</x:v>
       </x:c>
       <x:c r="B17" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A17)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A17)</x:f>
         <x:v>39</x:v>
       </x:c>
       <x:c r="C17" s="107" t="n">
         <x:f>B17/$A$5</x:f>
-        <x:v>0.07372400756143667</x:v>
+        <x:v>0.06989247311827956</x:v>
       </x:c>
       <x:c r="E17" s="37" t="str">
         <x:v>Machine Learning Street Talk</x:v>
       </x:c>
       <x:c r="F17" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E17)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E17)</x:f>
         <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="37" t="str">
-        <x:v>World Models</x:v>
+        <x:v>Computer Vision / 3D Vision</x:v>
       </x:c>
       <x:c r="B18" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A18)</x:f>
-        <x:v>34</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A18)</x:f>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C18" s="107" t="n">
         <x:f>B18/$A$5</x:f>
-        <x:v>0.06427221172022685</x:v>
+        <x:v>0.06451612903225806</x:v>
       </x:c>
       <x:c r="E18" s="37" t="str">
         <x:v>Microsoft Research</x:v>
       </x:c>
       <x:c r="F18" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E18)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E18)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="H18" s="71" t="str">
-        <x:v>The four priority areas contain 354 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
+        <x:v>The four priority areas contain 383 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
       </x:c>
       <x:c r="I18" s="71" t="str">
-        <x:v>The four priority areas contain 354 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
+        <x:v>The four priority areas contain 383 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
       </x:c>
       <x:c r="J18" s="71" t="str">
-        <x:v>The four priority areas contain 354 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
+        <x:v>The four priority areas contain 383 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
       </x:c>
       <x:c r="K18" s="71" t="str">
-        <x:v>The four priority areas contain 354 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
+        <x:v>The four priority areas contain 383 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
       </x:c>
       <x:c r="L18" s="71" t="str">
-        <x:v>The four priority areas contain 354 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
+        <x:v>The four priority areas contain 383 resources, meeting the initial 200+ target. Future fields can include thumbnails, subtitle languages, series relationships, and editorial notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="37" t="str">
-        <x:v>Computer Vision / 3D Vision</x:v>
+        <x:v>World Models</x:v>
       </x:c>
       <x:c r="B19" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A19)</x:f>
-        <x:v>33</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A19)</x:f>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C19" s="107" t="n">
         <x:f>B19/$A$5</x:f>
-        <x:v>0.062381852551984876</x:v>
+        <x:v>0.06093189964157706</x:v>
       </x:c>
       <x:c r="E19" s="37" t="str">
         <x:v>Stanford HAI</x:v>
       </x:c>
       <x:c r="F19" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E19)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E19)</x:f>
         <x:v>8</x:v>
       </x:c>
     </x:row>
@@ -1457,18 +1457,18 @@
         <x:v>World Models / Predictive Intelligence</x:v>
       </x:c>
       <x:c r="B20" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A20)</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A20)</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C20" s="107" t="n">
         <x:f>B20/$A$5</x:f>
-        <x:v>0.03780718336483932</x:v>
+        <x:v>0.03942652329749104</x:v>
       </x:c>
       <x:c r="E20" s="37" t="str">
         <x:v>No Priors: AI, Machine Learning, Tech, &amp; Startups</x:v>
       </x:c>
       <x:c r="F20" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E20)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E20)</x:f>
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1477,18 +1477,18 @@
         <x:v>Deep Learning Foundations</x:v>
       </x:c>
       <x:c r="B21" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A21)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A21)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="C21" s="107" t="n">
         <x:f>B21/$A$5</x:f>
-        <x:v>0.024574669187145556</x:v>
+        <x:v>0.023297491039426525</x:v>
       </x:c>
       <x:c r="E21" s="37" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
       <x:c r="F21" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E21)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E21)</x:f>
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1497,18 +1497,18 @@
         <x:v>AI Research Frontiers</x:v>
       </x:c>
       <x:c r="B22" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A22)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A22)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="C22" s="107" t="n">
         <x:f>B22/$A$5</x:f>
-        <x:v>0.020793950850661626</x:v>
+        <x:v>0.01971326164874552</x:v>
       </x:c>
       <x:c r="E22" s="37" t="str">
         <x:v>The Robot Brains Podcast</x:v>
       </x:c>
       <x:c r="F22" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E22)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E22)</x:f>
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1517,18 +1517,18 @@
         <x:v>AI Systems / Accelerated Computing</x:v>
       </x:c>
       <x:c r="B23" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A23)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A23)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="C23" s="107" t="n">
         <x:f>B23/$A$5</x:f>
-        <x:v>0.020793950850661626</x:v>
+        <x:v>0.01971326164874552</x:v>
       </x:c>
       <x:c r="E23" s="37" t="str">
         <x:v>The TWIML AI Podcast with Sam Charrington</x:v>
       </x:c>
       <x:c r="F23" s="78" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E23)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E23)</x:f>
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1537,18 +1537,18 @@
         <x:v>Computer Vision</x:v>
       </x:c>
       <x:c r="B24" s="85" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A24)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A24)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="C24" s="108" t="n">
         <x:f>B24/$A$5</x:f>
-        <x:v>0.01890359168241966</x:v>
+        <x:v>0.017921146953405017</x:v>
       </x:c>
       <x:c r="E24" s="40" t="str">
         <x:v>Berkeley RDI</x:v>
       </x:c>
       <x:c r="F24" s="80" t="n">
-        <x:f>COUNTIF('Resources'!$I$2:$I$530,E24)</x:f>
+        <x:f>COUNTIF('Resources'!$I$2:$I$559,E24)</x:f>
         <x:v>6</x:v>
       </x:c>
     </x:row>
@@ -34465,47 +34465,1845 @@
         <x:v>BV1sNSQByE5D</x:v>
       </x:c>
     </x:row>
+    <x:row r="531" ht="42" customHeight="1">
+      <x:c r="A531" s="21" t="str">
+        <x:v>ST-530</x:v>
+      </x:c>
+      <x:c r="B531" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C531" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D531" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E531" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Moonshot AI / Kimi</x:v>
+      </x:c>
+      <x:c r="F531" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G531" s="17" t="str">
+        <x:v>AGI Next 前沿峰会 | 月之暗面Kimi创始人杨植麟：Scaling Law、模型架构与Agent智能</x:v>
+      </x:c>
+      <x:c r="H531" s="17" t="str">
+        <x:v>Zhilin Yang</x:v>
+      </x:c>
+      <x:c r="I531" s="17" t="str">
+        <x:v>AITIME论道</x:v>
+      </x:c>
+      <x:c r="J531" s="22" t="str">
+        <x:v>Technical Keynote</x:v>
+      </x:c>
+      <x:c r="K531" s="23" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="L531" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1NxrHBgE6c</x:v>
+      </x:c>
+      <x:c r="M531" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N531" s="24" t="n">
+        <x:v>9207</x:v>
+      </x:c>
+      <x:c r="O531" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P531" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q531" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R531" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S531" s="17" t="str">
+        <x:v>Moonshot AI / Kimi. AGI Next keynote on scaling laws, model architecture, and agent intelligence.</x:v>
+      </x:c>
+      <x:c r="T531" s="16" t="str">
+        <x:v>BV1NxrHBgE6c</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="532" ht="42" customHeight="1">
+      <x:c r="A532" s="21" t="str">
+        <x:v>ST-531</x:v>
+      </x:c>
+      <x:c r="B532" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C532" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D532" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E532" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Moonshot AI / Kimi</x:v>
+      </x:c>
+      <x:c r="F532" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G532" s="17" t="str">
+        <x:v>杨植麟GTC完整演讲：Kimi如何重写大模型三大件</x:v>
+      </x:c>
+      <x:c r="H532" s="17" t="str">
+        <x:v>Zhilin Yang</x:v>
+      </x:c>
+      <x:c r="I532" s="17" t="str">
+        <x:v>opus精译</x:v>
+      </x:c>
+      <x:c r="J532" s="22" t="str">
+        <x:v>Conference Talk</x:v>
+      </x:c>
+      <x:c r="K532" s="23" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L532" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1RR3R6VEwy</x:v>
+      </x:c>
+      <x:c r="M532" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N532" s="24" t="n">
+        <x:v>5804</x:v>
+      </x:c>
+      <x:c r="O532" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P532" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q532" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R532" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S532" s="17" t="str">
+        <x:v>Moonshot AI / Kimi. Full GTC talk with Chinese translation; retained for its architecture and training-system detail.</x:v>
+      </x:c>
+      <x:c r="T532" s="16" t="str">
+        <x:v>BV1RR3R6VEwy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="533" ht="42" customHeight="1">
+      <x:c r="A533" s="21" t="str">
+        <x:v>ST-532</x:v>
+      </x:c>
+      <x:c r="B533" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C533" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D533" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E533" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / DeepSeek / High-Flyer</x:v>
+      </x:c>
+      <x:c r="F533" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G533" s="17" t="str">
+        <x:v>DeepSeek（幻方）早期内部采访视频</x:v>
+      </x:c>
+      <x:c r="H533" s="17" t="str">
+        <x:v>Wenfeng Liang and the High-Flyer team</x:v>
+      </x:c>
+      <x:c r="I533" s="17" t="str">
+        <x:v>i陆三金</x:v>
+      </x:c>
+      <x:c r="J533" s="22" t="str">
+        <x:v>Early Team Interview</x:v>
+      </x:c>
+      <x:c r="K533" s="23" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="L533" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1fSNFeTEUz</x:v>
+      </x:c>
+      <x:c r="M533" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N533" s="24" t="n">
+        <x:v>83871</x:v>
+      </x:c>
+      <x:c r="O533" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P533" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q533" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R533" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S533" s="17" t="str">
+        <x:v>DeepSeek / High-Flyer. Rare early internal interview footage from the High-Flyer team that later created DeepSeek.</x:v>
+      </x:c>
+      <x:c r="T533" s="16" t="str">
+        <x:v>BV1fSNFeTEUz</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="534" ht="42" customHeight="1">
+      <x:c r="A534" s="21" t="str">
+        <x:v>ST-533</x:v>
+      </x:c>
+      <x:c r="B534" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C534" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D534" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E534" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / DeepSeek</x:v>
+      </x:c>
+      <x:c r="F534" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G534" s="17" t="str">
+        <x:v>【专访一】DeepSeek梁文锋：中国硬核创新会越来越多</x:v>
+      </x:c>
+      <x:c r="H534" s="17" t="str">
+        <x:v>Wenfeng Liang</x:v>
+      </x:c>
+      <x:c r="I534" s="17" t="str">
+        <x:v>爱莲说Allie</x:v>
+      </x:c>
+      <x:c r="J534" s="22" t="str">
+        <x:v>Interview Adaptation</x:v>
+      </x:c>
+      <x:c r="K534" s="23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L534" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1gxffYTEsJ</x:v>
+      </x:c>
+      <x:c r="M534" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N534" s="24" t="n">
+        <x:v>224858</x:v>
+      </x:c>
+      <x:c r="O534" s="22" t="str">
+        <x:v>C | Community Selection</x:v>
+      </x:c>
+      <x:c r="P534" s="22" t="str">
+        <x:v>Reserve</x:v>
+      </x:c>
+      <x:c r="Q534" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R534" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S534" s="17" t="str">
+        <x:v>DeepSeek. Video adaptation of Wenfeng Liang's authorized Waves interview; useful primary remarks, but not an original filmed interview.</x:v>
+      </x:c>
+      <x:c r="T534" s="16" t="str">
+        <x:v>BV1gxffYTEsJ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="535" ht="42" customHeight="1">
+      <x:c r="A535" s="21" t="str">
+        <x:v>ST-534</x:v>
+      </x:c>
+      <x:c r="B535" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C535" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D535" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E535" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Alibaba Qwen</x:v>
+      </x:c>
+      <x:c r="F535" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G535" s="17" t="str">
+        <x:v>AGI-Next 前沿峰会 | 阿里Qwen技术负责人林俊旸：Towards a Generalist Agent</x:v>
+      </x:c>
+      <x:c r="H535" s="17" t="str">
+        <x:v>Junyang Lin</x:v>
+      </x:c>
+      <x:c r="I535" s="17" t="str">
+        <x:v>AITIME论道</x:v>
+      </x:c>
+      <x:c r="J535" s="22" t="str">
+        <x:v>Technical Keynote</x:v>
+      </x:c>
+      <x:c r="K535" s="23" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="L535" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1R1rHBxE2V</x:v>
+      </x:c>
+      <x:c r="M535" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N535" s="24" t="n">
+        <x:v>24960</x:v>
+      </x:c>
+      <x:c r="O535" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P535" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q535" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R535" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S535" s="17" t="str">
+        <x:v>Alibaba Qwen. AGI Next keynote on Qwen's path toward generalist agents.</x:v>
+      </x:c>
+      <x:c r="T535" s="16" t="str">
+        <x:v>BV1R1rHBxE2V</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="536" ht="42" customHeight="1">
+      <x:c r="A536" s="21" t="str">
+        <x:v>ST-535</x:v>
+      </x:c>
+      <x:c r="B536" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C536" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D536" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E536" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Alibaba Qwen</x:v>
+      </x:c>
+      <x:c r="F536" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G536" s="17" t="str">
+        <x:v>Qwen：通用模型之路-林俊旸</x:v>
+      </x:c>
+      <x:c r="H536" s="17" t="str">
+        <x:v>Junyang Lin</x:v>
+      </x:c>
+      <x:c r="I536" s="17" t="str">
+        <x:v>ModelScope官方账号</x:v>
+      </x:c>
+      <x:c r="J536" s="22" t="str">
+        <x:v>Technical Talk</x:v>
+      </x:c>
+      <x:c r="K536" s="23" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L536" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1wh3TzvE4k</x:v>
+      </x:c>
+      <x:c r="M536" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N536" s="24" t="n">
+        <x:v>3651</x:v>
+      </x:c>
+      <x:c r="O536" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P536" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q536" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R536" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S536" s="17" t="str">
+        <x:v>Alibaba Qwen. ModelScope-hosted technical overview of Qwen as a general-purpose model family.</x:v>
+      </x:c>
+      <x:c r="T536" s="16" t="str">
+        <x:v>BV1wh3TzvE4k</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="537" ht="42" customHeight="1">
+      <x:c r="A537" s="21" t="str">
+        <x:v>ST-536</x:v>
+      </x:c>
+      <x:c r="B537" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C537" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D537" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E537" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Alibaba Qwen</x:v>
+      </x:c>
+      <x:c r="F537" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G537" s="17" t="str">
+        <x:v>林俊旸详解Qwen模型设计中的每一次取舍 | 林俊旸 | Junyang Lin | 240703 | 原创中英字幕</x:v>
+      </x:c>
+      <x:c r="H537" s="17" t="str">
+        <x:v>Junyang Lin</x:v>
+      </x:c>
+      <x:c r="I537" s="17" t="str">
+        <x:v>京口先生</x:v>
+      </x:c>
+      <x:c r="J537" s="22" t="str">
+        <x:v>Technical Talk</x:v>
+      </x:c>
+      <x:c r="K537" s="23" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="L537" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1T3NuzvENT</x:v>
+      </x:c>
+      <x:c r="M537" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N537" s="24" t="n">
+        <x:v>32040</x:v>
+      </x:c>
+      <x:c r="O537" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P537" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q537" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R537" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S537" s="17" t="str">
+        <x:v>Alibaba Qwen. Long-form bilingual technical talk on the engineering choices behind Qwen.</x:v>
+      </x:c>
+      <x:c r="T537" s="16" t="str">
+        <x:v>BV1T3NuzvENT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="538" ht="42" customHeight="1">
+      <x:c r="A538" s="21" t="str">
+        <x:v>ST-537</x:v>
+      </x:c>
+      <x:c r="B538" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C538" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D538" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E538" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Tencent Hunyuan</x:v>
+      </x:c>
+      <x:c r="F538" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G538" s="17" t="str">
+        <x:v>腾讯混元大模型负责人王迪：揭秘万亿 MoE 系统工程之道｜智者访谈</x:v>
+      </x:c>
+      <x:c r="H538" s="17" t="str">
+        <x:v>Di Wang</x:v>
+      </x:c>
+      <x:c r="I538" s="17" t="str">
+        <x:v>机器之心官方</x:v>
+      </x:c>
+      <x:c r="J538" s="22" t="str">
+        <x:v>Technical Interview</x:v>
+      </x:c>
+      <x:c r="K538" s="23" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="L538" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1QuWae8Eoj</x:v>
+      </x:c>
+      <x:c r="M538" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N538" s="24" t="n">
+        <x:v>15271</x:v>
+      </x:c>
+      <x:c r="O538" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P538" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q538" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R538" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S538" s="17" t="str">
+        <x:v>Tencent Hunyuan. Machine Intelligence interview on the systems engineering of Hunyuan's trillion-parameter MoE model.</x:v>
+      </x:c>
+      <x:c r="T538" s="16" t="str">
+        <x:v>BV1QuWae8Eoj</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="539" ht="42" customHeight="1">
+      <x:c r="A539" s="21" t="str">
+        <x:v>ST-538</x:v>
+      </x:c>
+      <x:c r="B539" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C539" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D539" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E539" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Tencent Hunyuan</x:v>
+      </x:c>
+      <x:c r="F539" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G539" s="17" t="str">
+        <x:v>腾讯混元大模型发布会：超千亿参数、超2万亿Token的全链路自研大语言模型，混元大模型综合性能国内第一、诸多特性超越GPT3.5</x:v>
+      </x:c>
+      <x:c r="H539" s="17" t="str">
+        <x:v>Tencent Hunyuan team</x:v>
+      </x:c>
+      <x:c r="I539" s="17" t="str">
+        <x:v>创新指南针</x:v>
+      </x:c>
+      <x:c r="J539" s="22" t="str">
+        <x:v>Product and Technical Launch</x:v>
+      </x:c>
+      <x:c r="K539" s="23" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L539" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1rp4y1L7Hx</x:v>
+      </x:c>
+      <x:c r="M539" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N539" s="24" t="n">
+        <x:v>12547</x:v>
+      </x:c>
+      <x:c r="O539" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P539" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q539" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R539" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S539" s="17" t="str">
+        <x:v>Tencent Hunyuan. Full launch presentation covering Hunyuan's model, training stack, and deployment strategy.</x:v>
+      </x:c>
+      <x:c r="T539" s="16" t="str">
+        <x:v>BV1rp4y1L7Hx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="540" ht="42" customHeight="1">
+      <x:c r="A540" s="21" t="str">
+        <x:v>ST-539</x:v>
+      </x:c>
+      <x:c r="B540" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C540" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D540" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E540" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / MiniMax</x:v>
+      </x:c>
+      <x:c r="F540" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G540" s="17" t="str">
+        <x:v>【正片】MiniMax 创始人闫俊杰×罗永浩！大山并非无法翻越</x:v>
+      </x:c>
+      <x:c r="H540" s="17" t="str">
+        <x:v>Junjie Yan</x:v>
+      </x:c>
+      <x:c r="I540" s="17" t="str">
+        <x:v>罗永浩的十字路口</x:v>
+      </x:c>
+      <x:c r="J540" s="22" t="str">
+        <x:v>Long-form Video Interview</x:v>
+      </x:c>
+      <x:c r="K540" s="23" t="n">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="L540" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV11NmtBzE36</x:v>
+      </x:c>
+      <x:c r="M540" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N540" s="24" t="n">
+        <x:v>712316</x:v>
+      </x:c>
+      <x:c r="O540" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P540" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q540" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R540" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S540" s="17" t="str">
+        <x:v>MiniMax. Full long-form interview on MiniMax, model scaling, product strategy, and the path to advanced intelligence.</x:v>
+      </x:c>
+      <x:c r="T540" s="16" t="str">
+        <x:v>BV11NmtBzE36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="541" ht="42" customHeight="1">
+      <x:c r="A541" s="21" t="str">
+        <x:v>ST-540</x:v>
+      </x:c>
+      <x:c r="B541" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C541" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D541" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E541" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Zhipu AI</x:v>
+      </x:c>
+      <x:c r="F541" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G541" s="17" t="str">
+        <x:v>方略第十四期正片 | 方三文对话智谱CEO张鹏： 大模型不会只剩一家，多样性是技术革新的源动力</x:v>
+      </x:c>
+      <x:c r="H541" s="17" t="str">
+        <x:v>Peng Zhang</x:v>
+      </x:c>
+      <x:c r="I541" s="17" t="str">
+        <x:v>雪球官方账号</x:v>
+      </x:c>
+      <x:c r="J541" s="22" t="str">
+        <x:v>Long-form Video Interview</x:v>
+      </x:c>
+      <x:c r="K541" s="23" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="L541" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1zFPpzxECA</x:v>
+      </x:c>
+      <x:c r="M541" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N541" s="24" t="n">
+        <x:v>40534</x:v>
+      </x:c>
+      <x:c r="O541" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P541" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q541" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R541" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S541" s="17" t="str">
+        <x:v>Zhipu AI. Long-form conversation with Zhipu AI's CEO on model diversity and technology strategy.</x:v>
+      </x:c>
+      <x:c r="T541" s="16" t="str">
+        <x:v>BV1zFPpzxECA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="542" ht="42" customHeight="1">
+      <x:c r="A542" s="21" t="str">
+        <x:v>ST-541</x:v>
+      </x:c>
+      <x:c r="B542" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C542" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D542" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E542" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Zhipu AI</x:v>
+      </x:c>
+      <x:c r="F542" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G542" s="17" t="str">
+        <x:v>智谱唐杰：AGI 与 ChatGLM 之路</x:v>
+      </x:c>
+      <x:c r="H542" s="17" t="str">
+        <x:v>Jie Tang</x:v>
+      </x:c>
+      <x:c r="I542" s="17" t="str">
+        <x:v>西安数学张老师</x:v>
+      </x:c>
+      <x:c r="J542" s="22" t="str">
+        <x:v>Technical Talk</x:v>
+      </x:c>
+      <x:c r="K542" s="23" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="L542" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1KkPQznEVf</x:v>
+      </x:c>
+      <x:c r="M542" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N542" s="24" t="n">
+        <x:v>901</x:v>
+      </x:c>
+      <x:c r="O542" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P542" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q542" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R542" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S542" s="17" t="str">
+        <x:v>Zhipu AI. Technical and strategic talk on the road from ChatGLM toward AGI.</x:v>
+      </x:c>
+      <x:c r="T542" s="16" t="str">
+        <x:v>BV1KkPQznEVf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="543" ht="42" customHeight="1">
+      <x:c r="A543" s="21" t="str">
+        <x:v>ST-542</x:v>
+      </x:c>
+      <x:c r="B543" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C543" s="21" t="str">
+        <x:v>Vision</x:v>
+      </x:c>
+      <x:c r="D543" s="17" t="str">
+        <x:v>Computer Vision / 3D Vision</x:v>
+      </x:c>
+      <x:c r="E543" s="17" t="str">
+        <x:v>Multimodal Models / Computer Vision / Representation Learning / StepFun</x:v>
+      </x:c>
+      <x:c r="F543" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G543" s="17" t="str">
+        <x:v>攀登AGI的路径与实践万亿参数+多模融合- 姜大昕 阶跃星辰创始人CEO</x:v>
+      </x:c>
+      <x:c r="H543" s="17" t="str">
+        <x:v>Daxin Jiang</x:v>
+      </x:c>
+      <x:c r="I543" s="17" t="str">
+        <x:v>真豆组合包</x:v>
+      </x:c>
+      <x:c r="J543" s="22" t="str">
+        <x:v>Technical Keynote</x:v>
+      </x:c>
+      <x:c r="K543" s="23" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L543" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1ueB2YDEQc</x:v>
+      </x:c>
+      <x:c r="M543" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N543" s="24" t="n">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="O543" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P543" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q543" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R543" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S543" s="17" t="str">
+        <x:v>StepFun. Talk on trillion-parameter scaling and multimodal fusion at StepFun.</x:v>
+      </x:c>
+      <x:c r="T543" s="16" t="str">
+        <x:v>BV1ueB2YDEQc</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="544" ht="42" customHeight="1">
+      <x:c r="A544" s="21" t="str">
+        <x:v>ST-543</x:v>
+      </x:c>
+      <x:c r="B544" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C544" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D544" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E544" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / StepFun</x:v>
+      </x:c>
+      <x:c r="F544" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G544" s="17" t="str">
+        <x:v>【姜大昕博士 IEEE Fellow】大模型路径、实践与趋势</x:v>
+      </x:c>
+      <x:c r="H544" s="17" t="str">
+        <x:v>Daxin Jiang</x:v>
+      </x:c>
+      <x:c r="I544" s="17" t="str">
+        <x:v>AI开讲啦</x:v>
+      </x:c>
+      <x:c r="J544" s="22" t="str">
+        <x:v>Technical Talk</x:v>
+      </x:c>
+      <x:c r="K544" s="23" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="L544" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1vVr5BNEev</x:v>
+      </x:c>
+      <x:c r="M544" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N544" s="24" t="n">
+        <x:v>1064</x:v>
+      </x:c>
+      <x:c r="O544" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P544" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q544" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R544" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S544" s="17" t="str">
+        <x:v>StepFun. Focused technical overview of large-model paths, practice, and emerging trends.</x:v>
+      </x:c>
+      <x:c r="T544" s="16" t="str">
+        <x:v>BV1vVr5BNEev</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="545" ht="42" customHeight="1">
+      <x:c r="A545" s="21" t="str">
+        <x:v>ST-544</x:v>
+      </x:c>
+      <x:c r="B545" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C545" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D545" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E545" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Baichuan AI</x:v>
+      </x:c>
+      <x:c r="F545" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G545" s="17" t="str">
+        <x:v>【正片】对话王小川：造医生，战豆包，与无尽的 AI 非共识。【视频播客】</x:v>
+      </x:c>
+      <x:c r="H545" s="17" t="str">
+        <x:v>Xiaochuan Wang</x:v>
+      </x:c>
+      <x:c r="I545" s="17" t="str">
+        <x:v>硅基立场Pro</x:v>
+      </x:c>
+      <x:c r="J545" s="22" t="str">
+        <x:v>Long-form Video Interview</x:v>
+      </x:c>
+      <x:c r="K545" s="23" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="L545" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV19pLQ6VEBB</x:v>
+      </x:c>
+      <x:c r="M545" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N545" s="24" t="n">
+        <x:v>19226</x:v>
+      </x:c>
+      <x:c r="O545" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P545" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q545" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R545" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S545" s="17" t="str">
+        <x:v>Baichuan AI. Long-form interview on AI doctors, model competition, and Baichuan's non-consensus strategy.</x:v>
+      </x:c>
+      <x:c r="T545" s="16" t="str">
+        <x:v>BV19pLQ6VEBB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="546" ht="42" customHeight="1">
+      <x:c r="A546" s="21" t="str">
+        <x:v>ST-545</x:v>
+      </x:c>
+      <x:c r="B546" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C546" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D546" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E546" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Baichuan AI</x:v>
+      </x:c>
+      <x:c r="F546" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G546" s="17" t="str">
+        <x:v>【洪涛 百川联合创始人、总裁】百川智能：打造AGI时代的超级底座与应用</x:v>
+      </x:c>
+      <x:c r="H546" s="17" t="str">
+        <x:v>Tao Hong</x:v>
+      </x:c>
+      <x:c r="I546" s="17" t="str">
+        <x:v>AI开讲啦</x:v>
+      </x:c>
+      <x:c r="J546" s="22" t="str">
+        <x:v>Technical and Strategy Talk</x:v>
+      </x:c>
+      <x:c r="K546" s="23" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="L546" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1Yp4y1L7mp</x:v>
+      </x:c>
+      <x:c r="M546" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N546" s="24" t="n">
+        <x:v>1675</x:v>
+      </x:c>
+      <x:c r="O546" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P546" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q546" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R546" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S546" s="17" t="str">
+        <x:v>Baichuan AI. Talk by Baichuan's co-founder on foundation models and applications in the AGI era.</x:v>
+      </x:c>
+      <x:c r="T546" s="16" t="str">
+        <x:v>BV1Yp4y1L7mp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="547" ht="42" customHeight="1">
+      <x:c r="A547" s="21" t="str">
+        <x:v>ST-546</x:v>
+      </x:c>
+      <x:c r="B547" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C547" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D547" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E547" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / 01.AI</x:v>
+      </x:c>
+      <x:c r="F547" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G547" s="17" t="str">
+        <x:v>对谈李开复：AI越聪明，我们越该重新定义“有用”</x:v>
+      </x:c>
+      <x:c r="H547" s="17" t="str">
+        <x:v>Kai-Fu Lee</x:v>
+      </x:c>
+      <x:c r="I547" s="17" t="str">
+        <x:v>央视网</x:v>
+      </x:c>
+      <x:c r="J547" s="22" t="str">
+        <x:v>Broadcast Interview</x:v>
+      </x:c>
+      <x:c r="K547" s="23" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="L547" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1fUKG6SE1k</x:v>
+      </x:c>
+      <x:c r="M547" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N547" s="24" t="n">
+        <x:v>8494</x:v>
+      </x:c>
+      <x:c r="O547" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P547" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q547" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R547" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S547" s="17" t="str">
+        <x:v>01.AI. CCTV interview on how increasingly capable AI changes work, education, and the meaning of human usefulness.</x:v>
+      </x:c>
+      <x:c r="T547" s="16" t="str">
+        <x:v>BV1fUKG6SE1k</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="548" ht="42" customHeight="1">
+      <x:c r="A548" s="21" t="str">
+        <x:v>ST-547</x:v>
+      </x:c>
+      <x:c r="B548" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C548" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D548" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E548" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / 01.AI</x:v>
+      </x:c>
+      <x:c r="F548" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G548" s="17" t="str">
+        <x:v>20260718 刘润进化者 对谈李开复</x:v>
+      </x:c>
+      <x:c r="H548" s="17" t="str">
+        <x:v>Kai-Fu Lee</x:v>
+      </x:c>
+      <x:c r="I548" s="17" t="str">
+        <x:v>章振洋</x:v>
+      </x:c>
+      <x:c r="J548" s="22" t="str">
+        <x:v>Long-form Video Interview</x:v>
+      </x:c>
+      <x:c r="K548" s="23" t="n">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="L548" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1nvK66AEfz</x:v>
+      </x:c>
+      <x:c r="M548" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N548" s="24" t="n">
+        <x:v>3658</x:v>
+      </x:c>
+      <x:c r="O548" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P548" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q548" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R548" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S548" s="17" t="str">
+        <x:v>01.AI. Long-form 2026 conversation on AI models, applications, organizations, and entrepreneurship.</x:v>
+      </x:c>
+      <x:c r="T548" s="16" t="str">
+        <x:v>BV1nvK66AEfz</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="549" ht="42" customHeight="1">
+      <x:c r="A549" s="21" t="str">
+        <x:v>ST-548</x:v>
+      </x:c>
+      <x:c r="B549" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C549" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D549" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E549" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / 01.AI</x:v>
+      </x:c>
+      <x:c r="F549" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G549" s="17" t="str">
+        <x:v>2024北京智源大会 | 李开复&amp;张亚勤：通用人工智能-Fireside Chat</x:v>
+      </x:c>
+      <x:c r="H549" s="17" t="str">
+        <x:v>Kai-Fu Lee and Ya-Qin Zhang</x:v>
+      </x:c>
+      <x:c r="I549" s="17" t="str">
+        <x:v>账号已注销</x:v>
+      </x:c>
+      <x:c r="J549" s="22" t="str">
+        <x:v>Fireside Chat</x:v>
+      </x:c>
+      <x:c r="K549" s="23" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="L549" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1figseQEht</x:v>
+      </x:c>
+      <x:c r="M549" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N549" s="24" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="O549" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P549" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q549" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R549" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S549" s="17" t="str">
+        <x:v>01.AI. BAAI fireside chat on general artificial intelligence and China's model ecosystem.</x:v>
+      </x:c>
+      <x:c r="T549" s="16" t="str">
+        <x:v>BV1figseQEht</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="550" ht="42" customHeight="1">
+      <x:c r="A550" s="21" t="str">
+        <x:v>ST-549</x:v>
+      </x:c>
+      <x:c r="B550" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C550" s="21" t="str">
+        <x:v>Vision</x:v>
+      </x:c>
+      <x:c r="D550" s="17" t="str">
+        <x:v>Computer Vision / 3D Vision</x:v>
+      </x:c>
+      <x:c r="E550" s="17" t="str">
+        <x:v>Multimodal Models / Computer Vision / Representation Learning / ByteDance AI / Seed lineage</x:v>
+      </x:c>
+      <x:c r="F550" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G550" s="17" t="str">
+        <x:v>字节跳动曾妍：多粒度视觉语言预训练模型X-VLM</x:v>
+      </x:c>
+      <x:c r="H550" s="17" t="str">
+        <x:v>Yan Zeng</x:v>
+      </x:c>
+      <x:c r="I550" s="17" t="str">
+        <x:v>机器之心官方</x:v>
+      </x:c>
+      <x:c r="J550" s="22" t="str">
+        <x:v>Research Talk</x:v>
+      </x:c>
+      <x:c r="K550" s="23" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="L550" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1Da411S7jf</x:v>
+      </x:c>
+      <x:c r="M550" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N550" s="24" t="n">
+        <x:v>5153</x:v>
+      </x:c>
+      <x:c r="O550" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P550" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q550" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R550" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S550" s="17" t="str">
+        <x:v>ByteDance AI / Seed lineage. ByteDance research talk on X-VLM, an important multimodal predecessor in the research lineage that now continues in Seed.</x:v>
+      </x:c>
+      <x:c r="T550" s="16" t="str">
+        <x:v>BV1Da411S7jf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="551" ht="42" customHeight="1">
+      <x:c r="A551" s="21" t="str">
+        <x:v>ST-550</x:v>
+      </x:c>
+      <x:c r="B551" s="21" t="str">
+        <x:v>Course</x:v>
+      </x:c>
+      <x:c r="C551" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D551" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E551" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / ModelBest</x:v>
+      </x:c>
+      <x:c r="F551" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G551" s="17" t="str">
+        <x:v>【清华NLP】刘知远团队大模型公开课全网首发｜带你从入门到实战</x:v>
+      </x:c>
+      <x:c r="H551" s="17" t="str">
+        <x:v>Zhiyuan Liu and the Tsinghua NLP team</x:v>
+      </x:c>
+      <x:c r="I551" s="17" t="str">
+        <x:v>OpenBMB</x:v>
+      </x:c>
+      <x:c r="J551" s="22" t="str">
+        <x:v>Full Course / Tutorial Series</x:v>
+      </x:c>
+      <x:c r="K551" s="23" t="n">
+        <x:v>1057</x:v>
+      </x:c>
+      <x:c r="L551" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1UG411p7zv</x:v>
+      </x:c>
+      <x:c r="M551" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N551" s="24" t="n">
+        <x:v>659114</x:v>
+      </x:c>
+      <x:c r="O551" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P551" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q551" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R551" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S551" s="17" t="str">
+        <x:v>ModelBest. Substantial Tsinghua NLP course series led by ModelBest co-founder Zhiyuan Liu, spanning foundations through implementation.</x:v>
+      </x:c>
+      <x:c r="T551" s="16" t="str">
+        <x:v>BV1UG411p7zv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="552" ht="42" customHeight="1">
+      <x:c r="A552" s="21" t="str">
+        <x:v>ST-551</x:v>
+      </x:c>
+      <x:c r="B552" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C552" s="21" t="str">
+        <x:v>Robotics</x:v>
+      </x:c>
+      <x:c r="D552" s="17" t="str">
+        <x:v>Robotics / Embodied AI</x:v>
+      </x:c>
+      <x:c r="E552" s="17" t="str">
+        <x:v>Robot Learning / Embodied AI / Physical Intelligence / ModelBest</x:v>
+      </x:c>
+      <x:c r="F552" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G552" s="17" t="str">
+        <x:v>面壁CEO李大海：端侧智能如何叩开物理世界AGI大门？</x:v>
+      </x:c>
+      <x:c r="H552" s="17" t="str">
+        <x:v>Dahai Li</x:v>
+      </x:c>
+      <x:c r="I552" s="17" t="str">
+        <x:v>科技良友</x:v>
+      </x:c>
+      <x:c r="J552" s="22" t="str">
+        <x:v>Executive Talk</x:v>
+      </x:c>
+      <x:c r="K552" s="23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L552" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1nJEvzwEFU</x:v>
+      </x:c>
+      <x:c r="M552" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N552" s="24" t="n">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="O552" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P552" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q552" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R552" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S552" s="17" t="str">
+        <x:v>ModelBest. Concise talk on how on-device intelligence may connect digital models to physical-world AGI.</x:v>
+      </x:c>
+      <x:c r="T552" s="16" t="str">
+        <x:v>BV1nJEvzwEFU</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="553" ht="42" customHeight="1">
+      <x:c r="A553" s="21" t="str">
+        <x:v>ST-552</x:v>
+      </x:c>
+      <x:c r="B553" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C553" s="21" t="str">
+        <x:v>World Model</x:v>
+      </x:c>
+      <x:c r="D553" s="17" t="str">
+        <x:v>World Models / Predictive Intelligence</x:v>
+      </x:c>
+      <x:c r="E553" s="17" t="str">
+        <x:v>World Models / Video Generation / Spatial Intelligence / ShengShu Technology / Vidu</x:v>
+      </x:c>
+      <x:c r="F553" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G553" s="17" t="str">
+        <x:v>清华大学朱军教授：Generative AI: from Virtual to Physical World｜2025未来科学大奖周科学峰会【计算机科学专场】</x:v>
+      </x:c>
+      <x:c r="H553" s="17" t="str">
+        <x:v>Jun Zhu</x:v>
+      </x:c>
+      <x:c r="I553" s="17" t="str">
+        <x:v>未来论坛</x:v>
+      </x:c>
+      <x:c r="J553" s="22" t="str">
+        <x:v>Research Keynote</x:v>
+      </x:c>
+      <x:c r="K553" s="23" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="L553" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1sFcMzJE3X</x:v>
+      </x:c>
+      <x:c r="M553" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N553" s="24" t="n">
+        <x:v>2354</x:v>
+      </x:c>
+      <x:c r="O553" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P553" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q553" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R553" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S553" s="17" t="str">
+        <x:v>ShengShu Technology / Vidu. Research keynote tracing generative AI from virtual content toward physical-world modeling.</x:v>
+      </x:c>
+      <x:c r="T553" s="16" t="str">
+        <x:v>BV1sFcMzJE3X</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="554" ht="42" customHeight="1">
+      <x:c r="A554" s="21" t="str">
+        <x:v>ST-553</x:v>
+      </x:c>
+      <x:c r="B554" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C554" s="21" t="str">
+        <x:v>World Model</x:v>
+      </x:c>
+      <x:c r="D554" s="17" t="str">
+        <x:v>World Models / Predictive Intelligence</x:v>
+      </x:c>
+      <x:c r="E554" s="17" t="str">
+        <x:v>World Models / Video Generation / Spatial Intelligence / ShengShu Technology / Vidu</x:v>
+      </x:c>
+      <x:c r="F554" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G554" s="17" t="str">
+        <x:v>WAIC 2026 特别对话｜央视专访朱军：AI从生成视频，到理解世界</x:v>
+      </x:c>
+      <x:c r="H554" s="17" t="str">
+        <x:v>Jun Zhu</x:v>
+      </x:c>
+      <x:c r="I554" s="17" t="str">
+        <x:v>Vidu-AI</x:v>
+      </x:c>
+      <x:c r="J554" s="22" t="str">
+        <x:v>Broadcast Interview</x:v>
+      </x:c>
+      <x:c r="K554" s="23" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="L554" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1w3Kr6BEjm</x:v>
+      </x:c>
+      <x:c r="M554" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N554" s="24" t="n">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="O554" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P554" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q554" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R554" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S554" s="17" t="str">
+        <x:v>ShengShu Technology / Vidu. CCTV interview on moving from video generation toward general world models.</x:v>
+      </x:c>
+      <x:c r="T554" s="16" t="str">
+        <x:v>BV1w3Kr6BEjm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="555" ht="42" customHeight="1">
+      <x:c r="A555" s="21" t="str">
+        <x:v>ST-554</x:v>
+      </x:c>
+      <x:c r="B555" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C555" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D555" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E555" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Shanghai AI Laboratory</x:v>
+      </x:c>
+      <x:c r="F555" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G555" s="17" t="str">
+        <x:v>若AGI=通专融合，“它”是实现AGI的可行路径</x:v>
+      </x:c>
+      <x:c r="H555" s="17" t="str">
+        <x:v>Bowen Zhou</x:v>
+      </x:c>
+      <x:c r="I555" s="17" t="str">
+        <x:v>上海AILab</x:v>
+      </x:c>
+      <x:c r="J555" s="22" t="str">
+        <x:v>Invited Talk</x:v>
+      </x:c>
+      <x:c r="K555" s="23" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="L555" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV18M6FBEEJV</x:v>
+      </x:c>
+      <x:c r="M555" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N555" s="24" t="n">
+        <x:v>1283</x:v>
+      </x:c>
+      <x:c r="O555" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P555" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q555" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R555" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S555" s="17" t="str">
+        <x:v>Shanghai AI Laboratory. Official Shanghai AI Lab invited talk on combining general and specialized intelligence as a route to AGI.</x:v>
+      </x:c>
+      <x:c r="T555" s="16" t="str">
+        <x:v>BV18M6FBEEJV</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="556" ht="42" customHeight="1">
+      <x:c r="A556" s="21" t="str">
+        <x:v>ST-555</x:v>
+      </x:c>
+      <x:c r="B556" s="21" t="str">
+        <x:v>Course</x:v>
+      </x:c>
+      <x:c r="C556" s="21" t="str">
+        <x:v>Vision</x:v>
+      </x:c>
+      <x:c r="D556" s="17" t="str">
+        <x:v>Computer Vision / 3D Vision</x:v>
+      </x:c>
+      <x:c r="E556" s="17" t="str">
+        <x:v>Multimodal Models / Computer Vision / Representation Learning / Shanghai AI Laboratory / InternVL</x:v>
+      </x:c>
+      <x:c r="F556" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G556" s="17" t="str">
+        <x:v>【AI Talk 第五季01期】详解InternVL，开源多模态大模型“黑马”</x:v>
+      </x:c>
+      <x:c r="H556" s="17" t="str">
+        <x:v>InternVL team</x:v>
+      </x:c>
+      <x:c r="I556" s="17" t="str">
+        <x:v>OpenDataLab</x:v>
+      </x:c>
+      <x:c r="J556" s="22" t="str">
+        <x:v>Technical Tutorial</x:v>
+      </x:c>
+      <x:c r="K556" s="23" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="L556" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1Ur421T7qX</x:v>
+      </x:c>
+      <x:c r="M556" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N556" s="24" t="n">
+        <x:v>3671</x:v>
+      </x:c>
+      <x:c r="O556" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P556" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q556" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R556" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S556" s="17" t="str">
+        <x:v>Shanghai AI Laboratory / InternVL. Long technical deep dive into the InternVL open-source multimodal model family.</x:v>
+      </x:c>
+      <x:c r="T556" s="16" t="str">
+        <x:v>BV1Ur421T7qX</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="557" ht="42" customHeight="1">
+      <x:c r="A557" s="21" t="str">
+        <x:v>ST-556</x:v>
+      </x:c>
+      <x:c r="B557" s="21" t="str">
+        <x:v>Course</x:v>
+      </x:c>
+      <x:c r="C557" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D557" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E557" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Shanghai AI Laboratory / InternLM</x:v>
+      </x:c>
+      <x:c r="F557" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G557" s="17" t="str">
+        <x:v>书生·浦语大模型全链路开源体系</x:v>
+      </x:c>
+      <x:c r="H557" s="17" t="str">
+        <x:v>InternLM team</x:v>
+      </x:c>
+      <x:c r="I557" s="17" t="str">
+        <x:v>OpenMMLab</x:v>
+      </x:c>
+      <x:c r="J557" s="22" t="str">
+        <x:v>Technical Tutorial</x:v>
+      </x:c>
+      <x:c r="K557" s="23" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="L557" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1Vx421X72D</x:v>
+      </x:c>
+      <x:c r="M557" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N557" s="24" t="n">
+        <x:v>11309</x:v>
+      </x:c>
+      <x:c r="O557" s="22" t="str">
+        <x:v>A | Official / Original Creator / Organizer</x:v>
+      </x:c>
+      <x:c r="P557" s="22" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="Q557" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R557" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S557" s="17" t="str">
+        <x:v>Shanghai AI Laboratory / InternLM. Official tutorial on the open-source InternLM model and tooling stack.</x:v>
+      </x:c>
+      <x:c r="T557" s="16" t="str">
+        <x:v>BV1Vx421X72D</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="558" ht="42" customHeight="1">
+      <x:c r="A558" s="21" t="str">
+        <x:v>ST-557</x:v>
+      </x:c>
+      <x:c r="B558" s="21" t="str">
+        <x:v>Talk</x:v>
+      </x:c>
+      <x:c r="C558" s="21" t="str">
+        <x:v>Robotics</x:v>
+      </x:c>
+      <x:c r="D558" s="17" t="str">
+        <x:v>Robotics / Embodied AI</x:v>
+      </x:c>
+      <x:c r="E558" s="17" t="str">
+        <x:v>Robot Learning / Embodied AI / Physical Intelligence / Shanghai AI Laboratory</x:v>
+      </x:c>
+      <x:c r="F558" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G558" s="17" t="str">
+        <x:v>上海AI Lab最新！可泛化、可规模化的空间具身智能</x:v>
+      </x:c>
+      <x:c r="H558" s="17" t="str">
+        <x:v>Haoyi Zhu</x:v>
+      </x:c>
+      <x:c r="I558" s="17" t="str">
+        <x:v>3D视觉工坊</x:v>
+      </x:c>
+      <x:c r="J558" s="22" t="str">
+        <x:v>Research Talk</x:v>
+      </x:c>
+      <x:c r="K558" s="23" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="L558" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1FAMPzjEVX</x:v>
+      </x:c>
+      <x:c r="M558" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N558" s="24" t="n">
+        <x:v>2226</x:v>
+      </x:c>
+      <x:c r="O558" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P558" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q558" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R558" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S558" s="17" t="str">
+        <x:v>Shanghai AI Laboratory. Research talk on scalable spatial embodied intelligence, connecting 3D perception, world modeling, and robot learning.</x:v>
+      </x:c>
+      <x:c r="T558" s="16" t="str">
+        <x:v>BV1FAMPzjEVX</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="559" ht="42" customHeight="1">
+      <x:c r="A559" s="21" t="str">
+        <x:v>ST-558</x:v>
+      </x:c>
+      <x:c r="B559" s="21" t="str">
+        <x:v>Interview</x:v>
+      </x:c>
+      <x:c r="C559" s="21" t="str">
+        <x:v>Agent</x:v>
+      </x:c>
+      <x:c r="D559" s="17" t="str">
+        <x:v>Agents / Tool Use / Reasoning</x:v>
+      </x:c>
+      <x:c r="E559" s="17" t="str">
+        <x:v>Foundation Models / Agents / Reasoning / Tool Use / Moonshot AI / Zhipu AI / Baichuan AI / ModelBest</x:v>
+      </x:c>
+      <x:c r="F559" s="22" t="str">
+        <x:v>Chinese</x:v>
+      </x:c>
+      <x:c r="G559" s="17" t="str">
+        <x:v>2024智源大会-尖峰对话-通往AGI之路</x:v>
+      </x:c>
+      <x:c r="H559" s="17" t="str">
+        <x:v>Xiaochuan Wang, Peng Zhang, Zhilin Yang, and Dahai Li</x:v>
+      </x:c>
+      <x:c r="I559" s="17" t="str">
+        <x:v>啊是在想起我</x:v>
+      </x:c>
+      <x:c r="J559" s="22" t="str">
+        <x:v>Executive Panel</x:v>
+      </x:c>
+      <x:c r="K559" s="23" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="L559" s="16" t="str">
+        <x:v>https://www.bilibili.com/video/BV1BQGoemEMp</x:v>
+      </x:c>
+      <x:c r="M559" s="21" t="str">
+        <x:v>Bilibili</x:v>
+      </x:c>
+      <x:c r="N559" s="24" t="n">
+        <x:v>3768</x:v>
+      </x:c>
+      <x:c r="O559" s="22" t="str">
+        <x:v>B | University / Conference / Institution</x:v>
+      </x:c>
+      <x:c r="P559" s="22" t="str">
+        <x:v>Recommended</x:v>
+      </x:c>
+      <x:c r="Q559" s="22" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="R559" s="25" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="S559" s="17" t="str">
+        <x:v>Moonshot AI / Zhipu AI / Baichuan AI / ModelBest. BAAI 2024 panel bringing together four leading Chinese foundation-model CEOs on the road to AGI.</x:v>
+      </x:c>
+      <x:c r="T559" s="16" t="str">
+        <x:v>BV1BQGoemEMp</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="B2:B530">
+  <x:conditionalFormatting sqref="B2:B559">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Interview"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Course"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Talk"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="C2:C530">
+  <x:conditionalFormatting sqref="C2:C559">
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="World Model"/>
     <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Agent"/>
     <x:cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="Vision"/>
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Robotics"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="P2:P530">
+  <x:conditionalFormatting sqref="P2:P559">
     <x:cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="Core"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="Q2:Q530">
+  <x:conditionalFormatting sqref="Q2:Q559">
     <x:cfRule type="containsText" dxfId="8" priority="9" operator="containsText" text="Verified"/>
   </x:conditionalFormatting>
   <x:dataValidations count="6">
-    <x:dataValidation type="list" sqref="B2:B530">
+    <x:dataValidation type="list" sqref="B2:B559">
       <x:formula1>"Interview,Course,Talk"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C2:C530">
+    <x:dataValidation type="list" sqref="C2:C559">
       <x:formula1>"World Model,Agent,Vision,Robotics,Other"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="F2:F530">
+    <x:dataValidation type="list" sqref="F2:F559">
       <x:formula1>"Chinese,English,Bilingual"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="M2:M530">
+    <x:dataValidation type="list" sqref="M2:M559">
       <x:formula1>"YouTube,Bilibili,Xiaohongshu"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="P2:P530">
+    <x:dataValidation type="list" sqref="P2:P559">
       <x:formula1>"Core,Recommended,Reserve"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="Q2:Q530">
+    <x:dataValidation type="list" sqref="Q2:Q559">
       <x:formula1>"Verified,Pending Verification,Periodic Review,Inactive"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4e552cbb7174681"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9eed9e09bdf4c15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34607,31 +36405,31 @@
         <x:v>World Model</x:v>
       </x:c>
       <x:c r="B5" s="58" t="n">
-        <x:f>COUNTIF('Resources'!$C$2:$C$530,A5)</x:f>
-        <x:v>72</x:v>
+        <x:f>COUNTIF('Resources'!$C$2:$C$559,A5)</x:f>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C5" s="58" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A5,'Resources'!$B$2:$B$530,"Interview")</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A5,'Resources'!$B$2:$B$559,"Interview")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="58" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A5,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A5,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="E5" s="58" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A5,'Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A5,'Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F5" s="58" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A5,'Resources'!$M$2:$M$530,"YouTube")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A5,'Resources'!$M$2:$M$559,"YouTube")</x:f>
         <x:v>48</x:v>
       </x:c>
       <x:c r="G5" s="58" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A5,'Resources'!$M$2:$M$530,"Bilibili")</x:f>
-        <x:v>24</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A5,'Resources'!$M$2:$M$559,"Bilibili")</x:f>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="H5" s="59" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A5,'Resources'!$M$2:$M$530,"Xiaohongshu")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A5,'Resources'!$M$2:$M$559,"Xiaohongshu")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -34640,31 +36438,31 @@
         <x:v>Agent</x:v>
       </x:c>
       <x:c r="B6" s="60" t="n">
-        <x:f>COUNTIF('Resources'!$C$2:$C$530,A6)</x:f>
-        <x:v>83</x:v>
+        <x:f>COUNTIF('Resources'!$C$2:$C$559,A6)</x:f>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C6" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A6,'Resources'!$B$2:$B$530,"Interview")</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A6,'Resources'!$B$2:$B$559,"Interview")</x:f>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D6" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A6,'Resources'!$B$2:$B$530,"Course")</x:f>
-        <x:v>32</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A6,'Resources'!$B$2:$B$559,"Course")</x:f>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E6" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A6,'Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>29</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A6,'Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F6" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A6,'Resources'!$M$2:$M$530,"YouTube")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A6,'Resources'!$M$2:$M$559,"YouTube")</x:f>
         <x:v>52</x:v>
       </x:c>
       <x:c r="G6" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A6,'Resources'!$M$2:$M$530,"Bilibili")</x:f>
-        <x:v>31</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A6,'Resources'!$M$2:$M$559,"Bilibili")</x:f>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="H6" s="61" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A6,'Resources'!$M$2:$M$530,"Xiaohongshu")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A6,'Resources'!$M$2:$M$559,"Xiaohongshu")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -34673,31 +36471,31 @@
         <x:v>Vision</x:v>
       </x:c>
       <x:c r="B7" s="60" t="n">
-        <x:f>COUNTIF('Resources'!$C$2:$C$530,A7)</x:f>
-        <x:v>90</x:v>
+        <x:f>COUNTIF('Resources'!$C$2:$C$559,A7)</x:f>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C7" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A7,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A7,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D7" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A7,'Resources'!$B$2:$B$530,"Course")</x:f>
-        <x:v>44</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A7,'Resources'!$B$2:$B$559,"Course")</x:f>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E7" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A7,'Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>33</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A7,'Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A7,'Resources'!$M$2:$M$530,"YouTube")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A7,'Resources'!$M$2:$M$559,"YouTube")</x:f>
         <x:v>65</x:v>
       </x:c>
       <x:c r="G7" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A7,'Resources'!$M$2:$M$530,"Bilibili")</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A7,'Resources'!$M$2:$M$559,"Bilibili")</x:f>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="H7" s="61" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A7,'Resources'!$M$2:$M$530,"Xiaohongshu")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A7,'Resources'!$M$2:$M$559,"Xiaohongshu")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -34706,31 +36504,31 @@
         <x:v>Robotics</x:v>
       </x:c>
       <x:c r="B8" s="60" t="n">
-        <x:f>COUNTIF('Resources'!$C$2:$C$530,A8)</x:f>
-        <x:v>109</x:v>
+        <x:f>COUNTIF('Resources'!$C$2:$C$559,A8)</x:f>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="C8" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A8,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A8,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>28</x:v>
       </x:c>
       <x:c r="D8" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A8,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A8,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="E8" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A8,'Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>48</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A8,'Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F8" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A8,'Resources'!$M$2:$M$530,"YouTube")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A8,'Resources'!$M$2:$M$559,"YouTube")</x:f>
         <x:v>85</x:v>
       </x:c>
       <x:c r="G8" s="60" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A8,'Resources'!$M$2:$M$530,"Bilibili")</x:f>
-        <x:v>24</x:v>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A8,'Resources'!$M$2:$M$559,"Bilibili")</x:f>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="H8" s="61" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A8,'Resources'!$M$2:$M$530,"Xiaohongshu")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A8,'Resources'!$M$2:$M$559,"Xiaohongshu")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -34739,31 +36537,31 @@
         <x:v>Other</x:v>
       </x:c>
       <x:c r="B9" s="62" t="n">
-        <x:f>COUNTIF('Resources'!$C$2:$C$530,A9)</x:f>
+        <x:f>COUNTIF('Resources'!$C$2:$C$559,A9)</x:f>
         <x:v>175</x:v>
       </x:c>
       <x:c r="C9" s="62" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A9,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A9,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>52</x:v>
       </x:c>
       <x:c r="D9" s="62" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A9,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A9,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>66</x:v>
       </x:c>
       <x:c r="E9" s="62" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A9,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A9,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>57</x:v>
       </x:c>
       <x:c r="F9" s="62" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A9,'Resources'!$M$2:$M$530,"YouTube")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A9,'Resources'!$M$2:$M$559,"YouTube")</x:f>
         <x:v>175</x:v>
       </x:c>
       <x:c r="G9" s="62" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A9,'Resources'!$M$2:$M$530,"Bilibili")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A9,'Resources'!$M$2:$M$559,"Bilibili")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="63" t="n">
-        <x:f>COUNTIFS('Resources'!$C$2:$C$530,A9,'Resources'!$M$2:$M$530,"Xiaohongshu")</x:f>
+        <x:f>COUNTIFS('Resources'!$C$2:$C$559,A9,'Resources'!$M$2:$M$559,"Xiaohongshu")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -34827,7 +36625,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76fb057541cc4af2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda03dec0710646e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34865,19 +36663,19 @@
         <x:v>Agents</x:v>
       </x:c>
       <x:c r="B2" s="81" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A2)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A2)</x:f>
         <x:v>39</x:v>
       </x:c>
       <x:c r="C2" s="81" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A2,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A2,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D2" s="81" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A2,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A2,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="E2" s="82" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A2,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A2,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>13</x:v>
       </x:c>
     </x:row>
@@ -34886,20 +36684,20 @@
         <x:v>Agents / Tool Use / Reasoning</x:v>
       </x:c>
       <x:c r="B3" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A3)</x:f>
-        <x:v>41</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A3)</x:f>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C3" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A3,'Resources'!$B$2:$B$530,"Interview")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A3,'Resources'!$B$2:$B$559,"Interview")</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D3" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A3,'Resources'!$B$2:$B$530,"Course")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A3,'Resources'!$B$2:$B$559,"Course")</x:f>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E3" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A3,'Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A3,'Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -34907,19 +36705,19 @@
         <x:v>AI and Society</x:v>
       </x:c>
       <x:c r="B4" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A4)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A4)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C4" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A4,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A4,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D4" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A4,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A4,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E4" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A4,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A4,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -34928,19 +36726,19 @@
         <x:v>AI for Science</x:v>
       </x:c>
       <x:c r="B5" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A5)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A5)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A5,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A5,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A5,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A5,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E5" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A5,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A5,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -34949,19 +36747,19 @@
         <x:v>AI Foundations</x:v>
       </x:c>
       <x:c r="B6" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A6)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A6)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A6,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A6,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A6,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A6,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E6" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A6,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A6,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -34970,19 +36768,19 @@
         <x:v>AI Frontiers / Industry</x:v>
       </x:c>
       <x:c r="B7" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A7)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A7)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A7,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A7,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A7,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A7,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A7,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A7,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -34991,19 +36789,19 @@
         <x:v>AI Industry / Startups</x:v>
       </x:c>
       <x:c r="B8" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A8)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A8)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C8" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A8,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A8,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D8" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A8,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A8,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E8" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A8,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A8,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35012,19 +36810,19 @@
         <x:v>AI Research / Social Impact</x:v>
       </x:c>
       <x:c r="B9" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A9)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C9" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A9,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A9,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D9" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A9,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A9,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A9,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A9,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35033,19 +36831,19 @@
         <x:v>AI Research Frontiers</x:v>
       </x:c>
       <x:c r="B10" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A10)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A10)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="C10" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A10,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A10,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A10,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A10,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E10" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A10,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A10,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>11</x:v>
       </x:c>
     </x:row>
@@ -35054,19 +36852,19 @@
         <x:v>AI Startups / Foundation Models</x:v>
       </x:c>
       <x:c r="B11" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A11)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A11)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C11" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A11,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A11,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A11,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A11,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E11" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A11,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A11,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35075,19 +36873,19 @@
         <x:v>AI Systems / Accelerated Computing</x:v>
       </x:c>
       <x:c r="B12" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A12)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A12)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="C12" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A12,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A12,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D12" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A12,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A12,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A12,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A12,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -35096,19 +36894,19 @@
         <x:v>AI Systems / Infrastructure</x:v>
       </x:c>
       <x:c r="B13" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A13)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A13)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C13" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A13,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A13,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D13" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A13,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A13,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A13,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A13,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -35117,19 +36915,19 @@
         <x:v>Chinese AI Researchers / Industry</x:v>
       </x:c>
       <x:c r="B14" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A14)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A14)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C14" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A14,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A14,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D14" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A14,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A14,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A14,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A14,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35138,19 +36936,19 @@
         <x:v>Computer Vision</x:v>
       </x:c>
       <x:c r="B15" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A15)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A15)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="C15" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A15,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A15,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D15" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A15,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A15,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A15,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A15,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -35159,20 +36957,20 @@
         <x:v>Computer Vision / 3D Vision</x:v>
       </x:c>
       <x:c r="B16" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A16)</x:f>
-        <x:v>33</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A16)</x:f>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C16" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A16,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A16,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A16,'Resources'!$B$2:$B$530,"Course")</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A16,'Resources'!$B$2:$B$559,"Course")</x:f>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E16" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A16,'Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A16,'Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -35180,19 +36978,19 @@
         <x:v>Deep Learning / Representation Learning</x:v>
       </x:c>
       <x:c r="B17" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A17)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A17)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C17" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A17,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A17,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D17" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A17,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A17,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E17" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A17,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A17,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35201,19 +36999,19 @@
         <x:v>Deep Learning / Research Trends</x:v>
       </x:c>
       <x:c r="B18" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A18)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A18)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A18,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A18,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D18" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A18,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A18,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E18" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A18,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A18,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35222,19 +37020,19 @@
         <x:v>Deep Learning / Speech</x:v>
       </x:c>
       <x:c r="B19" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A19)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A19)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C19" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A19,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A19,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A19,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A19,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E19" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A19,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A19,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35243,19 +37041,19 @@
         <x:v>Deep Learning Foundations</x:v>
       </x:c>
       <x:c r="B20" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A20)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A20)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="C20" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A20,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A20,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D20" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A20,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A20,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="E20" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A20,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A20,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35264,19 +37062,19 @@
         <x:v>Deep Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B21" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A21)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A21)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C21" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A21,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A21,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D21" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A21,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A21,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E21" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A21,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A21,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35285,19 +37083,19 @@
         <x:v>Diffusion Models / Generative AI</x:v>
       </x:c>
       <x:c r="B22" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A22)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A22)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C22" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A22,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A22,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D22" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A22,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A22,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A22,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A22,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -35306,19 +37104,19 @@
         <x:v>Edge AI / TinyML</x:v>
       </x:c>
       <x:c r="B23" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A23)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A23)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C23" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A23,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A23,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D23" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A23,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A23,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E23" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A23,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A23,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35327,19 +37125,19 @@
         <x:v>Foundation Models / AI Frontiers</x:v>
       </x:c>
       <x:c r="B24" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A24)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A24)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C24" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A24,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A24,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D24" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A24,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A24,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E24" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A24,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A24,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -35348,19 +37146,19 @@
         <x:v>General AI / People</x:v>
       </x:c>
       <x:c r="B25" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A25)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A25)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C25" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A25,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A25,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D25" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A25,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A25,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E25" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A25,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A25,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35369,19 +37167,19 @@
         <x:v>Generative AI / Developers</x:v>
       </x:c>
       <x:c r="B26" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A26)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A26)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C26" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A26,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A26,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D26" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A26,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A26,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E26" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A26,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A26,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35390,19 +37188,19 @@
         <x:v>Graph Machine Learning</x:v>
       </x:c>
       <x:c r="B27" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A27)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A27)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C27" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A27,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A27,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D27" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A27,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A27,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E27" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A27,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A27,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -35411,19 +37209,19 @@
         <x:v>Large-Model Systems</x:v>
       </x:c>
       <x:c r="B28" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A28)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A28)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C28" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A28,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A28,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D28" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A28,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A28,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E28" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A28,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A28,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -35432,19 +37230,19 @@
         <x:v>Machine Learning / Engineering Practice</x:v>
       </x:c>
       <x:c r="B29" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A29)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A29)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C29" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A29,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A29,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D29" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A29,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A29,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E29" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A29,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A29,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35453,19 +37251,19 @@
         <x:v>Machine Learning Foundations</x:v>
       </x:c>
       <x:c r="B30" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A30)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A30)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C30" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A30,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A30,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D30" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A30,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A30,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E30" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A30,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A30,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35474,19 +37272,19 @@
         <x:v>Machine Learning Frontiers</x:v>
       </x:c>
       <x:c r="B31" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A31)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A31)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A31,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A31,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D31" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A31,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A31,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E31" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A31,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A31,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>8</x:v>
       </x:c>
     </x:row>
@@ -35495,19 +37293,19 @@
         <x:v>Machine Learning Research</x:v>
       </x:c>
       <x:c r="B32" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A32)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A32)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C32" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A32,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A32,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D32" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A32,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A32,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E32" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A32,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A32,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -35516,19 +37314,19 @@
         <x:v>MLOps / AI Product Engineering</x:v>
       </x:c>
       <x:c r="B33" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A33)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A33)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C33" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A33,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A33,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D33" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A33,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A33,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E33" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A33,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A33,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35537,19 +37335,19 @@
         <x:v>MLOps / Applied AI</x:v>
       </x:c>
       <x:c r="B34" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A34)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A34)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C34" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A34,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A34,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D34" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A34,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A34,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E34" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A34,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A34,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35558,19 +37356,19 @@
         <x:v>Multimodal Learning</x:v>
       </x:c>
       <x:c r="B35" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A35)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A35)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C35" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A35,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A35,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D35" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A35,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A35,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E35" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A35,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A35,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -35579,19 +37377,19 @@
         <x:v>Natural Language Processing</x:v>
       </x:c>
       <x:c r="B36" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A36)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A36)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A36,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A36,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D36" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A36,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A36,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E36" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A36,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A36,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -35600,19 +37398,19 @@
         <x:v>Natural Language Processing / Transformers</x:v>
       </x:c>
       <x:c r="B37" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A37)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A37)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C37" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A37,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A37,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D37" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A37,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A37,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E37" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A37,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A37,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35621,19 +37419,19 @@
         <x:v>Neural Network Foundations</x:v>
       </x:c>
       <x:c r="B38" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A38)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A38)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C38" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A38,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A38,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D38" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A38,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A38,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E38" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A38,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A38,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35642,19 +37440,19 @@
         <x:v>Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B39" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A39)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A39)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C39" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A39,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A39,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D39" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A39,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A39,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E39" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A39,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A39,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35663,19 +37461,19 @@
         <x:v>Representation Learning / Generative Models</x:v>
       </x:c>
       <x:c r="B40" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A40)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A40)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="C40" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A40,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A40,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D40" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A40,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A40,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E40" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A40,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A40,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -35684,19 +37482,19 @@
         <x:v>Robotics</x:v>
       </x:c>
       <x:c r="B41" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A41)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A41)</x:f>
         <x:v>42</x:v>
       </x:c>
       <x:c r="C41" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A41,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A41,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D41" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A41,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A41,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="E41" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A41,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A41,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>14</x:v>
       </x:c>
     </x:row>
@@ -35705,20 +37503,20 @@
         <x:v>Robotics / Embodied AI</x:v>
       </x:c>
       <x:c r="B42" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A42)</x:f>
-        <x:v>67</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A42)</x:f>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C42" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A42,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A42,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D42" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A42,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A42,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="E42" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A42,'Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>36</x:v>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A42,'Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -35726,19 +37524,19 @@
         <x:v>Transformers / Large Models</x:v>
       </x:c>
       <x:c r="B43" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A43)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A43)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C43" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A43,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A43,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D43" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A43,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A43,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E43" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A43,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A43,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35747,19 +37545,19 @@
         <x:v>Trustworthy AI / Safety</x:v>
       </x:c>
       <x:c r="B44" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A44)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A44)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C44" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A44,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A44,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D44" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A44,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A44,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E44" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A44,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A44,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -35768,19 +37566,19 @@
         <x:v>Vision</x:v>
       </x:c>
       <x:c r="B45" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A45)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A45)</x:f>
         <x:v>39</x:v>
       </x:c>
       <x:c r="C45" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A45,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A45,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="D45" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A45,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A45,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="E45" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A45,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A45,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>14</x:v>
       </x:c>
     </x:row>
@@ -35789,19 +37587,19 @@
         <x:v>World Models</x:v>
       </x:c>
       <x:c r="B46" s="83" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A46)</x:f>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A46)</x:f>
         <x:v>34</x:v>
       </x:c>
       <x:c r="C46" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A46,'Resources'!$B$2:$B$530,"Interview")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A46,'Resources'!$B$2:$B$559,"Interview")</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D46" s="83" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A46,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A46,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="E46" s="84" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A46,'Resources'!$B$2:$B$530,"Talk")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A46,'Resources'!$B$2:$B$559,"Talk")</x:f>
         <x:v>12</x:v>
       </x:c>
     </x:row>
@@ -35810,26 +37608,26 @@
         <x:v>World Models / Predictive Intelligence</x:v>
       </x:c>
       <x:c r="B47" s="85" t="n">
-        <x:f>COUNTIF('Resources'!$D$2:$D$530,A47)</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTIF('Resources'!$D$2:$D$559,A47)</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C47" s="85" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A47,'Resources'!$B$2:$B$530,"Interview")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A47,'Resources'!$B$2:$B$559,"Interview")</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D47" s="85" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A47,'Resources'!$B$2:$B$530,"Course")</x:f>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A47,'Resources'!$B$2:$B$559,"Course")</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="E47" s="86" t="n">
-        <x:f>COUNTIFS('Resources'!$D$2:$D$530,A47,'Resources'!$B$2:$B$530,"Talk")</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTIFS('Resources'!$D$2:$D$559,A47,'Resources'!$B$2:$B$559,"Talk")</x:f>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R911563c7685d429f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dd5fffd36214081"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat: group recurring interview series
</commit_message>
<xml_diff>
--- a/data/scholar_tube_seed_list.xlsx
+++ b/data/scholar_tube_seed_list.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2e0d03c5733e4aa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="2" r:id="Rcd43c82167ed44b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Areas" sheetId="3" r:id="R3f55f99ef6804033"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Index" sheetId="4" r:id="Rcce263b1d2b84387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="5" r:id="R84d3185298ef4875"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4052dc09d37f4f49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="2" r:id="Ref17d8ad2b1c44fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Areas" sheetId="3" r:id="Ra710be06f1ff400f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Index" sheetId="4" r:id="R78de0de059b0423a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="5" r:id="R6d92465872b549e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1066,40 +1066,40 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="B2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="C2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="D2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="E2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="F2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="G2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="H2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="I2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="J2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="K2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
       <x:c r="L2" s="32" t="str">
-        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Course series: 25 | Metadata checked: 2026-08-12</x:v>
+        <x:v>Curated resources: 546 direct video links | Four priority areas: 371 | Series: 40 (25 course, 15 interview) | Metadata checked: 2026-08-12</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
@@ -1427,19 +1427,19 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H18" s="73" t="str">
-        <x:v>25 explicit course series group 80 videos into 137 course entries. Individual canonical links remain available in the Resources sheet.</x:v>
+        <x:v>25 course series group 80 videos into 137 course entries; 15 interview series groups 82 episodes into 80 interview entries. Individual canonical links remain available in Resources.</x:v>
       </x:c>
       <x:c r="I18" s="73" t="str">
-        <x:v>25 explicit course series group 80 videos into 137 course entries. Individual canonical links remain available in the Resources sheet.</x:v>
+        <x:v>25 course series group 80 videos into 137 course entries; 15 interview series groups 82 episodes into 80 interview entries. Individual canonical links remain available in Resources.</x:v>
       </x:c>
       <x:c r="J18" s="73" t="str">
-        <x:v>25 explicit course series group 80 videos into 137 course entries. Individual canonical links remain available in the Resources sheet.</x:v>
+        <x:v>25 course series group 80 videos into 137 course entries; 15 interview series groups 82 episodes into 80 interview entries. Individual canonical links remain available in Resources.</x:v>
       </x:c>
       <x:c r="K18" s="73" t="str">
-        <x:v>25 explicit course series group 80 videos into 137 course entries. Individual canonical links remain available in the Resources sheet.</x:v>
+        <x:v>25 course series group 80 videos into 137 course entries; 15 interview series groups 82 episodes into 80 interview entries. Individual canonical links remain available in Resources.</x:v>
       </x:c>
       <x:c r="L18" s="73" t="str">
-        <x:v>25 explicit course series group 80 videos into 137 course entries. Individual canonical links remain available in the Resources sheet.</x:v>
+        <x:v>25 course series group 80 videos into 137 course entries; 15 interview series groups 82 episodes into 80 interview entries. Individual canonical links remain available in Resources.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1750,9 +1750,15 @@
       <x:c r="T2" s="16" t="str">
         <x:v>cdiD-9MMpb0</x:v>
       </x:c>
-      <x:c r="U2" s="17" t="str"/>
-      <x:c r="V2" s="27"/>
-      <x:c r="W2" s="17" t="str"/>
+      <x:c r="U2" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V2" s="27" t="n">
+        <x:v>20221029</x:v>
+      </x:c>
+      <x:c r="W2" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="22" t="str">
@@ -1815,9 +1821,15 @@
       <x:c r="T3" s="16" t="str">
         <x:v>NNr6gPelJ3E</x:v>
       </x:c>
-      <x:c r="U3" s="17" t="str"/>
-      <x:c r="V3" s="27"/>
-      <x:c r="W3" s="17" t="str"/>
+      <x:c r="U3" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V3" s="27" t="n">
+        <x:v>20240602</x:v>
+      </x:c>
+      <x:c r="W3" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="22" t="str">
@@ -1880,9 +1892,15 @@
       <x:c r="T4" s="16" t="str">
         <x:v>vif8NQcjVf0</x:v>
       </x:c>
-      <x:c r="U4" s="17" t="str"/>
-      <x:c r="V4" s="27"/>
-      <x:c r="W4" s="17" t="str"/>
+      <x:c r="U4" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V4" s="27" t="n">
+        <x:v>20260323</x:v>
+      </x:c>
+      <x:c r="W4" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="22" t="str">
@@ -1945,9 +1963,15 @@
       <x:c r="T5" s="16" t="str">
         <x:v>AaTRHFaaPG8</x:v>
       </x:c>
-      <x:c r="U5" s="17" t="str"/>
-      <x:c r="V5" s="27"/>
-      <x:c r="W5" s="17" t="str"/>
+      <x:c r="U5" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V5" s="27" t="n">
+        <x:v>20230330</x:v>
+      </x:c>
+      <x:c r="W5" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="22" t="str">
@@ -2010,9 +2034,15 @@
       <x:c r="T6" s="16" t="str">
         <x:v>cQ48rP_Rs4g</x:v>
       </x:c>
-      <x:c r="U6" s="17" t="str"/>
-      <x:c r="V6" s="27"/>
-      <x:c r="W6" s="17" t="str"/>
+      <x:c r="U6" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V6" s="27" t="n">
+        <x:v>20190715</x:v>
+      </x:c>
+      <x:c r="W6" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="22" t="str">
@@ -2075,9 +2105,15 @@
       <x:c r="T7" s="16" t="str">
         <x:v>-HzgcbRXUK8</x:v>
       </x:c>
-      <x:c r="U7" s="17" t="str"/>
-      <x:c r="V7" s="27"/>
-      <x:c r="W7" s="17" t="str"/>
+      <x:c r="U7" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V7" s="27" t="n">
+        <x:v>20250723</x:v>
+      </x:c>
+      <x:c r="W7" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="22" t="str">
@@ -2140,9 +2176,15 @@
       <x:c r="T8" s="16" t="str">
         <x:v>hppbxV9C63g</x:v>
       </x:c>
-      <x:c r="U8" s="17" t="str"/>
-      <x:c r="V8" s="27"/>
-      <x:c r="W8" s="17" t="str"/>
+      <x:c r="U8" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V8" s="27" t="n">
+        <x:v>20220714</x:v>
+      </x:c>
+      <x:c r="W8" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="22" t="str">
@@ -2205,9 +2247,15 @@
       <x:c r="T9" s="16" t="str">
         <x:v>aR20FWCCjAs</x:v>
       </x:c>
-      <x:c r="U9" s="17" t="str"/>
-      <x:c r="V9" s="27"/>
-      <x:c r="W9" s="17" t="str"/>
+      <x:c r="U9" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V9" s="27" t="n">
+        <x:v>20251125</x:v>
+      </x:c>
+      <x:c r="W9" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="22" t="str">
@@ -2270,9 +2318,15 @@
       <x:c r="T10" s="16" t="str">
         <x:v>lXUZvyajciY</x:v>
       </x:c>
-      <x:c r="U10" s="17" t="str"/>
-      <x:c r="V10" s="27"/>
-      <x:c r="W10" s="17" t="str"/>
+      <x:c r="U10" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V10" s="27" t="n">
+        <x:v>20251017</x:v>
+      </x:c>
+      <x:c r="W10" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="22" t="str">
@@ -2335,9 +2389,15 @@
       <x:c r="T11" s="16" t="str">
         <x:v>n1E9IZfvGMA</x:v>
       </x:c>
-      <x:c r="U11" s="17" t="str"/>
-      <x:c r="V11" s="27"/>
-      <x:c r="W11" s="17" t="str"/>
+      <x:c r="U11" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V11" s="27" t="n">
+        <x:v>20260213</x:v>
+      </x:c>
+      <x:c r="W11" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="22" t="str">
@@ -2400,9 +2460,15 @@
       <x:c r="T12" s="16" t="str">
         <x:v>21EYKqUsPfg</x:v>
       </x:c>
-      <x:c r="U12" s="17" t="str"/>
-      <x:c r="V12" s="27"/>
-      <x:c r="W12" s="17" t="str"/>
+      <x:c r="U12" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V12" s="27" t="n">
+        <x:v>20250926</x:v>
+      </x:c>
+      <x:c r="W12" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="22" t="str">
@@ -2465,9 +2531,15 @@
       <x:c r="T13" s="16" t="str">
         <x:v>mDG_Hx3BSUE</x:v>
       </x:c>
-      <x:c r="U13" s="17" t="str"/>
-      <x:c r="V13" s="27"/>
-      <x:c r="W13" s="17" t="str"/>
+      <x:c r="U13" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V13" s="27" t="n">
+        <x:v>20260313</x:v>
+      </x:c>
+      <x:c r="W13" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="22" t="str">
@@ -2530,9 +2602,15 @@
       <x:c r="T14" s="16" t="str">
         <x:v>Yf1o0TQzry8</x:v>
       </x:c>
-      <x:c r="U14" s="17" t="str"/>
-      <x:c r="V14" s="27"/>
-      <x:c r="W14" s="17" t="str"/>
+      <x:c r="U14" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V14" s="27" t="n">
+        <x:v>20230327</x:v>
+      </x:c>
+      <x:c r="W14" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="22" t="str">
@@ -2595,9 +2673,15 @@
       <x:c r="T15" s="16" t="str">
         <x:v>pE3KKUKXcTM</x:v>
       </x:c>
-      <x:c r="U15" s="17" t="str"/>
-      <x:c r="V15" s="27"/>
-      <x:c r="W15" s="17" t="str"/>
+      <x:c r="U15" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V15" s="27" t="n">
+        <x:v>20241002</x:v>
+      </x:c>
+      <x:c r="W15" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="22" t="str">
@@ -2660,9 +2744,15 @@
       <x:c r="T16" s="16" t="str">
         <x:v>a42key59cZQ</x:v>
       </x:c>
-      <x:c r="U16" s="17" t="str"/>
-      <x:c r="V16" s="27"/>
-      <x:c r="W16" s="17" t="str"/>
+      <x:c r="U16" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V16" s="27" t="n">
+        <x:v>20241113</x:v>
+      </x:c>
+      <x:c r="W16" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="22" t="str">
@@ -2855,9 +2945,15 @@
       <x:c r="T19" s="16" t="str">
         <x:v>nUtwOUNoZw0</x:v>
       </x:c>
-      <x:c r="U19" s="17" t="str"/>
-      <x:c r="V19" s="27"/>
-      <x:c r="W19" s="17" t="str"/>
+      <x:c r="U19" s="17" t="str">
+        <x:v>The Robot Brains Podcast</x:v>
+      </x:c>
+      <x:c r="V19" s="27" t="n">
+        <x:v>20210805</x:v>
+      </x:c>
+      <x:c r="W19" s="17" t="str">
+        <x:v>robot-brains-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="22" t="str">
@@ -2985,9 +3081,15 @@
       <x:c r="T21" s="16" t="str">
         <x:v>cFNI2FORAc0</x:v>
       </x:c>
-      <x:c r="U21" s="17" t="str"/>
-      <x:c r="V21" s="27"/>
-      <x:c r="W21" s="17" t="str"/>
+      <x:c r="U21" s="17" t="str">
+        <x:v>Latent Space Interviews</x:v>
+      </x:c>
+      <x:c r="V21" s="27" t="n">
+        <x:v>20260603</x:v>
+      </x:c>
+      <x:c r="W21" s="17" t="str">
+        <x:v>latent-space-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="22" t="str">
@@ -3115,9 +3217,15 @@
       <x:c r="T23" s="16" t="str">
         <x:v>98O-QxW2Xoo</x:v>
       </x:c>
-      <x:c r="U23" s="17" t="str"/>
-      <x:c r="V23" s="27"/>
-      <x:c r="W23" s="17" t="str"/>
+      <x:c r="U23" s="17" t="str">
+        <x:v>Weights &amp; Biases Interviews</x:v>
+      </x:c>
+      <x:c r="V23" s="27" t="n">
+        <x:v>20230518</x:v>
+      </x:c>
+      <x:c r="W23" s="17" t="str">
+        <x:v>weights-and-biases-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="22" t="str">
@@ -3180,9 +3288,15 @@
       <x:c r="T24" s="16" t="str">
         <x:v>2wprKvXnErE</x:v>
       </x:c>
-      <x:c r="U24" s="17" t="str"/>
-      <x:c r="V24" s="27"/>
-      <x:c r="W24" s="17" t="str"/>
+      <x:c r="U24" s="17" t="str">
+        <x:v>Weights &amp; Biases Interviews</x:v>
+      </x:c>
+      <x:c r="V24" s="27" t="n">
+        <x:v>20230713</x:v>
+      </x:c>
+      <x:c r="W24" s="17" t="str">
+        <x:v>weights-and-biases-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="22" t="str">
@@ -3245,9 +3359,15 @@
       <x:c r="T25" s="16" t="str">
         <x:v>AHOw0huInzs</x:v>
       </x:c>
-      <x:c r="U25" s="17" t="str"/>
-      <x:c r="V25" s="27"/>
-      <x:c r="W25" s="17" t="str"/>
+      <x:c r="U25" s="17" t="str">
+        <x:v>The Robot Brains Podcast</x:v>
+      </x:c>
+      <x:c r="V25" s="27" t="n">
+        <x:v>20210724</x:v>
+      </x:c>
+      <x:c r="W25" s="17" t="str">
+        <x:v>robot-brains-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="22" t="str">
@@ -3310,9 +3430,15 @@
       <x:c r="T26" s="16" t="str">
         <x:v>sD24pZh7pmQ</x:v>
       </x:c>
-      <x:c r="U26" s="17" t="str"/>
-      <x:c r="V26" s="27"/>
-      <x:c r="W26" s="17" t="str"/>
+      <x:c r="U26" s="17" t="str">
+        <x:v>Weights &amp; Biases Interviews</x:v>
+      </x:c>
+      <x:c r="V26" s="27" t="n">
+        <x:v>20230420</x:v>
+      </x:c>
+      <x:c r="W26" s="17" t="str">
+        <x:v>weights-and-biases-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="22" t="str">
@@ -3375,9 +3501,15 @@
       <x:c r="T27" s="16" t="str">
         <x:v>LdMydLBDgEQ</x:v>
       </x:c>
-      <x:c r="U27" s="17" t="str"/>
-      <x:c r="V27" s="27"/>
-      <x:c r="W27" s="17" t="str"/>
+      <x:c r="U27" s="17" t="str">
+        <x:v>Weights &amp; Biases Interviews</x:v>
+      </x:c>
+      <x:c r="V27" s="27" t="n">
+        <x:v>20230302</x:v>
+      </x:c>
+      <x:c r="W27" s="17" t="str">
+        <x:v>weights-and-biases-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="22" t="str">
@@ -3505,9 +3637,15 @@
       <x:c r="T29" s="16" t="str">
         <x:v>1dYThQgOyZU</x:v>
       </x:c>
-      <x:c r="U29" s="17" t="str"/>
-      <x:c r="V29" s="27"/>
-      <x:c r="W29" s="17" t="str"/>
+      <x:c r="U29" s="17" t="str">
+        <x:v>No Priors</x:v>
+      </x:c>
+      <x:c r="V29" s="27" t="n">
+        <x:v>20260312</x:v>
+      </x:c>
+      <x:c r="W29" s="17" t="str">
+        <x:v>no-priors-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="22" t="str">
@@ -3635,9 +3773,15 @@
       <x:c r="T31" s="16" t="str">
         <x:v>Vu5nKPRZRDs</x:v>
       </x:c>
-      <x:c r="U31" s="17" t="str"/>
-      <x:c r="V31" s="27"/>
-      <x:c r="W31" s="17" t="str"/>
+      <x:c r="U31" s="17" t="str">
+        <x:v>Stanford Medicine AI in Life Sciences Symposium</x:v>
+      </x:c>
+      <x:c r="V31" s="27" t="n">
+        <x:v>20260610</x:v>
+      </x:c>
+      <x:c r="W31" s="17" t="str">
+        <x:v>stanford-medicine-ai-life-sciences-symposium</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="22" t="str">
@@ -3700,9 +3844,15 @@
       <x:c r="T32" s="16" t="str">
         <x:v>kwSVtQ7dziU</x:v>
       </x:c>
-      <x:c r="U32" s="17" t="str"/>
-      <x:c r="V32" s="27"/>
-      <x:c r="W32" s="17" t="str"/>
+      <x:c r="U32" s="17" t="str">
+        <x:v>No Priors</x:v>
+      </x:c>
+      <x:c r="V32" s="27" t="n">
+        <x:v>20260320</x:v>
+      </x:c>
+      <x:c r="W32" s="17" t="str">
+        <x:v>no-priors-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="22" t="str">
@@ -3765,9 +3915,15 @@
       <x:c r="T33" s="16" t="str">
         <x:v>hhq9cYqz1-Y</x:v>
       </x:c>
-      <x:c r="U33" s="17" t="str"/>
-      <x:c r="V33" s="27"/>
-      <x:c r="W33" s="17" t="str"/>
+      <x:c r="U33" s="17" t="str">
+        <x:v>Stanford Medicine AI in Life Sciences Symposium</x:v>
+      </x:c>
+      <x:c r="V33" s="27" t="n">
+        <x:v>20260610</x:v>
+      </x:c>
+      <x:c r="W33" s="17" t="str">
+        <x:v>stanford-medicine-ai-life-sciences-symposium</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="22" t="str">
@@ -3830,9 +3986,15 @@
       <x:c r="T34" s="16" t="str">
         <x:v>tYGMfd3_D1o</x:v>
       </x:c>
-      <x:c r="U34" s="17" t="str"/>
-      <x:c r="V34" s="27"/>
-      <x:c r="W34" s="17" t="str"/>
+      <x:c r="U34" s="17" t="str">
+        <x:v>Eye on AI</x:v>
+      </x:c>
+      <x:c r="V34" s="27" t="n">
+        <x:v>20230510</x:v>
+      </x:c>
+      <x:c r="W34" s="17" t="str">
+        <x:v>eye-on-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="22" t="str">
@@ -3895,9 +4057,15 @@
       <x:c r="T35" s="16" t="str">
         <x:v>rMSEqJ_4EBk</x:v>
       </x:c>
-      <x:c r="U35" s="17" t="str"/>
-      <x:c r="V35" s="27"/>
-      <x:c r="W35" s="17" t="str"/>
+      <x:c r="U35" s="17" t="str">
+        <x:v>Machine Learning Street Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V35" s="27" t="n">
+        <x:v>20251021</x:v>
+      </x:c>
+      <x:c r="W35" s="17" t="str">
+        <x:v>machine-learning-street-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="22" t="str">
@@ -3960,9 +4128,15 @@
       <x:c r="T36" s="16" t="str">
         <x:v>rLG68k2blOc</x:v>
       </x:c>
-      <x:c r="U36" s="17" t="str"/>
-      <x:c r="V36" s="27"/>
-      <x:c r="W36" s="17" t="str"/>
+      <x:c r="U36" s="17" t="str">
+        <x:v>The Robot Brains Podcast</x:v>
+      </x:c>
+      <x:c r="V36" s="27" t="n">
+        <x:v>20230510</x:v>
+      </x:c>
+      <x:c r="W36" s="17" t="str">
+        <x:v>robot-brains-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="22" t="str">
@@ -4025,9 +4199,15 @@
       <x:c r="T37" s="16" t="str">
         <x:v>kuvFoXzTK3E</x:v>
       </x:c>
-      <x:c r="U37" s="17" t="str"/>
-      <x:c r="V37" s="27"/>
-      <x:c r="W37" s="17" t="str"/>
+      <x:c r="U37" s="17" t="str">
+        <x:v>Machine Learning Street Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V37" s="27" t="n">
+        <x:v>20240410</x:v>
+      </x:c>
+      <x:c r="W37" s="17" t="str">
+        <x:v>machine-learning-street-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="22" t="str">
@@ -4090,9 +4270,15 @@
       <x:c r="T38" s="16" t="str">
         <x:v>V_VXOdf1NMw</x:v>
       </x:c>
-      <x:c r="U38" s="17" t="str"/>
-      <x:c r="V38" s="27"/>
-      <x:c r="W38" s="17" t="str"/>
+      <x:c r="U38" s="17" t="str">
+        <x:v>Machine Learning Street Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V38" s="27" t="n">
+        <x:v>20230311</x:v>
+      </x:c>
+      <x:c r="W38" s="17" t="str">
+        <x:v>machine-learning-street-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="22" t="str">
@@ -4155,9 +4341,15 @@
       <x:c r="T39" s="16" t="str">
         <x:v>fCoavgGZ64Y</x:v>
       </x:c>
-      <x:c r="U39" s="17" t="str"/>
-      <x:c r="V39" s="27"/>
-      <x:c r="W39" s="17" t="str"/>
+      <x:c r="U39" s="17" t="str">
+        <x:v>The Robot Brains Podcast</x:v>
+      </x:c>
+      <x:c r="V39" s="27" t="n">
+        <x:v>20210921</x:v>
+      </x:c>
+      <x:c r="W39" s="17" t="str">
+        <x:v>robot-brains-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="22" t="str">
@@ -4220,9 +4412,15 @@
       <x:c r="T40" s="16" t="str">
         <x:v>DtePicx_kFY</x:v>
       </x:c>
-      <x:c r="U40" s="17" t="str"/>
-      <x:c r="V40" s="27"/>
-      <x:c r="W40" s="17" t="str"/>
+      <x:c r="U40" s="17" t="str">
+        <x:v>Machine Learning Street Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V40" s="27" t="n">
+        <x:v>20251123</x:v>
+      </x:c>
+      <x:c r="W40" s="17" t="str">
+        <x:v>machine-learning-street-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="22" t="str">
@@ -4285,9 +4483,15 @@
       <x:c r="T41" s="16" t="str">
         <x:v>hM_h0UA7upI</x:v>
       </x:c>
-      <x:c r="U41" s="17" t="str"/>
-      <x:c r="V41" s="27"/>
-      <x:c r="W41" s="17" t="str"/>
+      <x:c r="U41" s="17" t="str">
+        <x:v>No Priors</x:v>
+      </x:c>
+      <x:c r="V41" s="27" t="n">
+        <x:v>20240905</x:v>
+      </x:c>
+      <x:c r="W41" s="17" t="str">
+        <x:v>no-priors-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="22" t="str">
@@ -4350,9 +4554,15 @@
       <x:c r="T42" s="16" t="str">
         <x:v>pIbIZ_Bxl_g</x:v>
       </x:c>
-      <x:c r="U42" s="17" t="str"/>
-      <x:c r="V42" s="27"/>
-      <x:c r="W42" s="17" t="str"/>
+      <x:c r="U42" s="17" t="str">
+        <x:v>Latent Space Interviews</x:v>
+      </x:c>
+      <x:c r="V42" s="27" t="n">
+        <x:v>20250819</x:v>
+      </x:c>
+      <x:c r="W42" s="17" t="str">
+        <x:v>latent-space-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="22" t="str">
@@ -4415,9 +4625,15 @@
       <x:c r="T43" s="16" t="str">
         <x:v>URtF_UHYBSo</x:v>
       </x:c>
-      <x:c r="U43" s="17" t="str"/>
-      <x:c r="V43" s="27"/>
-      <x:c r="W43" s="17" t="str"/>
+      <x:c r="U43" s="17" t="str">
+        <x:v>Machine Learning Street Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V43" s="27" t="n">
+        <x:v>20241103</x:v>
+      </x:c>
+      <x:c r="W43" s="17" t="str">
+        <x:v>machine-learning-street-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="22" t="str">
@@ -4480,9 +4696,15 @@
       <x:c r="T44" s="16" t="str">
         <x:v>HhGOGuJY1Wk</x:v>
       </x:c>
-      <x:c r="U44" s="17" t="str"/>
-      <x:c r="V44" s="27"/>
-      <x:c r="W44" s="17" t="str"/>
+      <x:c r="U44" s="17" t="str">
+        <x:v>Weights &amp; Biases Interviews</x:v>
+      </x:c>
+      <x:c r="V44" s="27" t="n">
+        <x:v>20230105</x:v>
+      </x:c>
+      <x:c r="W44" s="17" t="str">
+        <x:v>weights-and-biases-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="22" t="str">
@@ -4545,9 +4767,15 @@
       <x:c r="T45" s="16" t="str">
         <x:v>AREWYbVtX64</x:v>
       </x:c>
-      <x:c r="U45" s="17" t="str"/>
-      <x:c r="V45" s="27"/>
-      <x:c r="W45" s="17" t="str"/>
+      <x:c r="U45" s="17" t="str">
+        <x:v>Machine Learning Street Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V45" s="27" t="n">
+        <x:v>20260520</x:v>
+      </x:c>
+      <x:c r="W45" s="17" t="str">
+        <x:v>machine-learning-street-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="22" t="str">
@@ -4610,9 +4838,15 @@
       <x:c r="T46" s="16" t="str">
         <x:v>86ib0sfdFtw</x:v>
       </x:c>
-      <x:c r="U46" s="17" t="str"/>
-      <x:c r="V46" s="27"/>
-      <x:c r="W46" s="17" t="str"/>
+      <x:c r="U46" s="17" t="str">
+        <x:v>Machine Learning Street Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V46" s="27" t="n">
+        <x:v>20220104</x:v>
+      </x:c>
+      <x:c r="W46" s="17" t="str">
+        <x:v>machine-learning-street-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="22" t="str">
@@ -4675,9 +4909,15 @@
       <x:c r="T47" s="16" t="str">
         <x:v>k-xtmISBCNE</x:v>
       </x:c>
-      <x:c r="U47" s="17" t="str"/>
-      <x:c r="V47" s="27"/>
-      <x:c r="W47" s="17" t="str"/>
+      <x:c r="U47" s="17" t="str">
+        <x:v>No Priors</x:v>
+      </x:c>
+      <x:c r="V47" s="27" t="n">
+        <x:v>20260108</x:v>
+      </x:c>
+      <x:c r="W47" s="17" t="str">
+        <x:v>no-priors-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="22" t="str">
@@ -4740,9 +4980,15 @@
       <x:c r="T48" s="16" t="str">
         <x:v>KKUKikuV58o</x:v>
       </x:c>
-      <x:c r="U48" s="17" t="str"/>
-      <x:c r="V48" s="27"/>
-      <x:c r="W48" s="17" t="str"/>
+      <x:c r="U48" s="17" t="str">
+        <x:v>Machine Learning Street Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V48" s="27" t="n">
+        <x:v>20250706</x:v>
+      </x:c>
+      <x:c r="W48" s="17" t="str">
+        <x:v>machine-learning-street-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="22" t="str">
@@ -4805,9 +5051,15 @@
       <x:c r="T49" s="16" t="str">
         <x:v>asCgCv2XB4s</x:v>
       </x:c>
-      <x:c r="U49" s="17" t="str"/>
-      <x:c r="V49" s="27"/>
-      <x:c r="W49" s="17" t="str"/>
+      <x:c r="U49" s="17" t="str">
+        <x:v>No Priors</x:v>
+      </x:c>
+      <x:c r="V49" s="27" t="n">
+        <x:v>20260618</x:v>
+      </x:c>
+      <x:c r="W49" s="17" t="str">
+        <x:v>no-priors-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
       <x:c r="A50" s="22" t="str">
@@ -4870,9 +5122,15 @@
       <x:c r="T50" s="16" t="str">
         <x:v>5mY71rGXAkM</x:v>
       </x:c>
-      <x:c r="U50" s="17" t="str"/>
-      <x:c r="V50" s="27"/>
-      <x:c r="W50" s="17" t="str"/>
+      <x:c r="U50" s="17" t="str">
+        <x:v>The TWIML AI Podcast</x:v>
+      </x:c>
+      <x:c r="V50" s="27" t="n">
+        <x:v>20250217</x:v>
+      </x:c>
+      <x:c r="W50" s="17" t="str">
+        <x:v>twiml-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
       <x:c r="A51" s="22" t="str">
@@ -5000,9 +5258,15 @@
       <x:c r="T52" s="16" t="str">
         <x:v>Yp_u1NpbkJg</x:v>
       </x:c>
-      <x:c r="U52" s="17" t="str"/>
-      <x:c r="V52" s="27"/>
-      <x:c r="W52" s="17" t="str"/>
+      <x:c r="U52" s="17" t="str">
+        <x:v>Latent Space Interviews</x:v>
+      </x:c>
+      <x:c r="V52" s="27" t="n">
+        <x:v>20260624</x:v>
+      </x:c>
+      <x:c r="W52" s="17" t="str">
+        <x:v>latent-space-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
       <x:c r="A53" s="22" t="str">
@@ -5065,9 +5329,15 @@
       <x:c r="T53" s="16" t="str">
         <x:v>2SWRU7YOd6c</x:v>
       </x:c>
-      <x:c r="U53" s="17" t="str"/>
-      <x:c r="V53" s="27"/>
-      <x:c r="W53" s="17" t="str"/>
+      <x:c r="U53" s="17" t="str">
+        <x:v>No Priors</x:v>
+      </x:c>
+      <x:c r="V53" s="27" t="n">
+        <x:v>20240522</x:v>
+      </x:c>
+      <x:c r="W53" s="17" t="str">
+        <x:v>no-priors-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
       <x:c r="A54" s="22" t="str">
@@ -5130,9 +5400,15 @@
       <x:c r="T54" s="16" t="str">
         <x:v>PlLmdTcsAWU</x:v>
       </x:c>
-      <x:c r="U54" s="17" t="str"/>
-      <x:c r="V54" s="27"/>
-      <x:c r="W54" s="17" t="str"/>
+      <x:c r="U54" s="17" t="str">
+        <x:v>The Robot Brains Podcast</x:v>
+      </x:c>
+      <x:c r="V54" s="27" t="n">
+        <x:v>20210921</x:v>
+      </x:c>
+      <x:c r="W54" s="17" t="str">
+        <x:v>robot-brains-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
       <x:c r="A55" s="22" t="str">
@@ -5195,9 +5471,15 @@
       <x:c r="T55" s="16" t="str">
         <x:v>tNNFJa5pUEg</x:v>
       </x:c>
-      <x:c r="U55" s="17" t="str"/>
-      <x:c r="V55" s="27"/>
-      <x:c r="W55" s="17" t="str"/>
+      <x:c r="U55" s="17" t="str">
+        <x:v>No Priors</x:v>
+      </x:c>
+      <x:c r="V55" s="27" t="n">
+        <x:v>20260417</x:v>
+      </x:c>
+      <x:c r="W55" s="17" t="str">
+        <x:v>no-priors-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
       <x:c r="A56" s="22" t="str">
@@ -5260,9 +5542,15 @@
       <x:c r="T56" s="16" t="str">
         <x:v>YE1UDwksAOc</x:v>
       </x:c>
-      <x:c r="U56" s="17" t="str"/>
-      <x:c r="V56" s="27"/>
-      <x:c r="W56" s="17" t="str"/>
+      <x:c r="U56" s="17" t="str">
+        <x:v>The Robot Brains Podcast</x:v>
+      </x:c>
+      <x:c r="V56" s="27" t="n">
+        <x:v>20210817</x:v>
+      </x:c>
+      <x:c r="W56" s="17" t="str">
+        <x:v>robot-brains-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
       <x:c r="A57" s="22" t="str">
@@ -5325,9 +5613,15 @@
       <x:c r="T57" s="16" t="str">
         <x:v>35ZWesLrv5A</x:v>
       </x:c>
-      <x:c r="U57" s="17" t="str"/>
-      <x:c r="V57" s="27"/>
-      <x:c r="W57" s="17" t="str"/>
+      <x:c r="U57" s="17" t="str">
+        <x:v>Latent Space Interviews</x:v>
+      </x:c>
+      <x:c r="V57" s="27" t="n">
+        <x:v>20250815</x:v>
+      </x:c>
+      <x:c r="W57" s="17" t="str">
+        <x:v>latent-space-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
       <x:c r="A58" s="22" t="str">
@@ -5455,9 +5749,15 @@
       <x:c r="T59" s="16" t="str">
         <x:v>k_Wrd1kI1B0</x:v>
       </x:c>
-      <x:c r="U59" s="17" t="str"/>
-      <x:c r="V59" s="27"/>
-      <x:c r="W59" s="17" t="str"/>
+      <x:c r="U59" s="17" t="str">
+        <x:v>The Robot Brains Podcast</x:v>
+      </x:c>
+      <x:c r="V59" s="27" t="n">
+        <x:v>20230816</x:v>
+      </x:c>
+      <x:c r="W59" s="17" t="str">
+        <x:v>robot-brains-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
       <x:c r="A60" s="22" t="str">
@@ -5520,9 +5820,15 @@
       <x:c r="T60" s="16" t="str">
         <x:v>oNKt1yhY4GY</x:v>
       </x:c>
-      <x:c r="U60" s="17" t="str"/>
-      <x:c r="V60" s="27"/>
-      <x:c r="W60" s="17" t="str"/>
+      <x:c r="U60" s="17" t="str">
+        <x:v>The TWIML AI Podcast</x:v>
+      </x:c>
+      <x:c r="V60" s="27" t="n">
+        <x:v>20250331</x:v>
+      </x:c>
+      <x:c r="W60" s="17" t="str">
+        <x:v>twiml-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
       <x:c r="A61" s="22" t="str">
@@ -5585,9 +5891,15 @@
       <x:c r="T61" s="16" t="str">
         <x:v>m2VqaNKstGc</x:v>
       </x:c>
-      <x:c r="U61" s="17" t="str"/>
-      <x:c r="V61" s="27"/>
-      <x:c r="W61" s="17" t="str"/>
+      <x:c r="U61" s="17" t="str">
+        <x:v>Latent Space Interviews</x:v>
+      </x:c>
+      <x:c r="V61" s="27" t="n">
+        <x:v>20250403</x:v>
+      </x:c>
+      <x:c r="W61" s="17" t="str">
+        <x:v>latent-space-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="42" customHeight="1">
       <x:c r="A62" s="22" t="str">
@@ -5650,9 +5962,15 @@
       <x:c r="T62" s="16" t="str">
         <x:v>I5xsDMJMdwo</x:v>
       </x:c>
-      <x:c r="U62" s="17" t="str"/>
-      <x:c r="V62" s="27"/>
-      <x:c r="W62" s="17" t="str"/>
+      <x:c r="U62" s="17" t="str">
+        <x:v>Eye on AI</x:v>
+      </x:c>
+      <x:c r="V62" s="27" t="n">
+        <x:v>20230412</x:v>
+      </x:c>
+      <x:c r="W62" s="17" t="str">
+        <x:v>eye-on-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
       <x:c r="A63" s="22" t="str">
@@ -5715,9 +6033,15 @@
       <x:c r="T63" s="16" t="str">
         <x:v>9mvZHd3TMa8</x:v>
       </x:c>
-      <x:c r="U63" s="17" t="str"/>
-      <x:c r="V63" s="27"/>
-      <x:c r="W63" s="17" t="str"/>
+      <x:c r="U63" s="17" t="str">
+        <x:v>The TWIML AI Podcast</x:v>
+      </x:c>
+      <x:c r="V63" s="27" t="n">
+        <x:v>20180917</x:v>
+      </x:c>
+      <x:c r="W63" s="17" t="str">
+        <x:v>twiml-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="42" customHeight="1">
       <x:c r="A64" s="22" t="str">
@@ -5780,9 +6104,15 @@
       <x:c r="T64" s="16" t="str">
         <x:v>HQucglw-4t8</x:v>
       </x:c>
-      <x:c r="U64" s="17" t="str"/>
-      <x:c r="V64" s="27"/>
-      <x:c r="W64" s="17" t="str"/>
+      <x:c r="U64" s="17" t="str">
+        <x:v>Latent Space Interviews</x:v>
+      </x:c>
+      <x:c r="V64" s="27" t="n">
+        <x:v>20251108</x:v>
+      </x:c>
+      <x:c r="W64" s="17" t="str">
+        <x:v>latent-space-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="42" customHeight="1">
       <x:c r="A65" s="22" t="str">
@@ -5845,9 +6175,15 @@
       <x:c r="T65" s="16" t="str">
         <x:v>y7k50Qux9Hc</x:v>
       </x:c>
-      <x:c r="U65" s="17" t="str"/>
-      <x:c r="V65" s="27"/>
-      <x:c r="W65" s="17" t="str"/>
+      <x:c r="U65" s="17" t="str">
+        <x:v>Weights &amp; Biases Interviews</x:v>
+      </x:c>
+      <x:c r="V65" s="27" t="n">
+        <x:v>20230410</x:v>
+      </x:c>
+      <x:c r="W65" s="17" t="str">
+        <x:v>weights-and-biases-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="42" customHeight="1">
       <x:c r="A66" s="22" t="str">
@@ -5910,9 +6246,15 @@
       <x:c r="T66" s="16" t="str">
         <x:v>C8SuqeH_Mg0</x:v>
       </x:c>
-      <x:c r="U66" s="17" t="str"/>
-      <x:c r="V66" s="27"/>
-      <x:c r="W66" s="17" t="str"/>
+      <x:c r="U66" s="17" t="str">
+        <x:v>The TWIML AI Podcast</x:v>
+      </x:c>
+      <x:c r="V66" s="27" t="n">
+        <x:v>20220509</x:v>
+      </x:c>
+      <x:c r="W66" s="17" t="str">
+        <x:v>twiml-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="42" customHeight="1">
       <x:c r="A67" s="22" t="str">
@@ -5975,9 +6317,15 @@
       <x:c r="T67" s="16" t="str">
         <x:v>PtZGHdDdWmY</x:v>
       </x:c>
-      <x:c r="U67" s="17" t="str"/>
-      <x:c r="V67" s="27"/>
-      <x:c r="W67" s="17" t="str"/>
+      <x:c r="U67" s="17" t="str">
+        <x:v>Eye on AI</x:v>
+      </x:c>
+      <x:c r="V67" s="27" t="n">
+        <x:v>20241023</x:v>
+      </x:c>
+      <x:c r="W67" s="17" t="str">
+        <x:v>eye-on-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="42" customHeight="1">
       <x:c r="A68" s="22" t="str">
@@ -6040,9 +6388,15 @@
       <x:c r="T68" s="16" t="str">
         <x:v>VIZwxufxg28</x:v>
       </x:c>
-      <x:c r="U68" s="17" t="str"/>
-      <x:c r="V68" s="27"/>
-      <x:c r="W68" s="17" t="str"/>
+      <x:c r="U68" s="17" t="str">
+        <x:v>The TWIML AI Podcast</x:v>
+      </x:c>
+      <x:c r="V68" s="27" t="n">
+        <x:v>20240527</x:v>
+      </x:c>
+      <x:c r="W68" s="17" t="str">
+        <x:v>twiml-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="42" customHeight="1">
       <x:c r="A69" s="22" t="str">
@@ -6105,9 +6459,15 @@
       <x:c r="T69" s="16" t="str">
         <x:v>uJ4l0awqAYA</x:v>
       </x:c>
-      <x:c r="U69" s="17" t="str"/>
-      <x:c r="V69" s="27"/>
-      <x:c r="W69" s="17" t="str"/>
+      <x:c r="U69" s="17" t="str">
+        <x:v>The TWIML AI Podcast</x:v>
+      </x:c>
+      <x:c r="V69" s="27" t="n">
+        <x:v>20200430</x:v>
+      </x:c>
+      <x:c r="W69" s="17" t="str">
+        <x:v>twiml-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="42" customHeight="1">
       <x:c r="A70" s="22" t="str">
@@ -6170,9 +6530,15 @@
       <x:c r="T70" s="16" t="str">
         <x:v>Pb_dJ6nUeBE</x:v>
       </x:c>
-      <x:c r="U70" s="17" t="str"/>
-      <x:c r="V70" s="27"/>
-      <x:c r="W70" s="17" t="str"/>
+      <x:c r="U70" s="17" t="str">
+        <x:v>The TWIML AI Podcast</x:v>
+      </x:c>
+      <x:c r="V70" s="27" t="n">
+        <x:v>20230605</x:v>
+      </x:c>
+      <x:c r="W70" s="17" t="str">
+        <x:v>twiml-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="42" customHeight="1">
       <x:c r="A71" s="22" t="str">
@@ -6235,9 +6601,15 @@
       <x:c r="T71" s="16" t="str">
         <x:v>eTzhu0wEF3o</x:v>
       </x:c>
-      <x:c r="U71" s="17" t="str"/>
-      <x:c r="V71" s="27"/>
-      <x:c r="W71" s="17" t="str"/>
+      <x:c r="U71" s="17" t="str">
+        <x:v>Eye on AI</x:v>
+      </x:c>
+      <x:c r="V71" s="27" t="n">
+        <x:v>20240109</x:v>
+      </x:c>
+      <x:c r="W71" s="17" t="str">
+        <x:v>eye-on-ai-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="42" customHeight="1">
       <x:c r="A72" s="22" t="str">
@@ -6495,9 +6867,15 @@
       <x:c r="T75" s="16" t="str">
         <x:v>SYuSZIIYOfI</x:v>
       </x:c>
-      <x:c r="U75" s="17" t="str"/>
-      <x:c r="V75" s="27"/>
-      <x:c r="W75" s="17" t="str"/>
+      <x:c r="U75" s="17" t="str">
+        <x:v>硅谷101｜AI Conversations</x:v>
+      </x:c>
+      <x:c r="V75" s="27" t="n">
+        <x:v>20260306</x:v>
+      </x:c>
+      <x:c r="W75" s="17" t="str">
+        <x:v>silicon-valley-101-ai-conversations</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="42" customHeight="1">
       <x:c r="A76" s="22" t="str">
@@ -16729,9 +17107,15 @@
       <x:c r="T227" s="16" t="str">
         <x:v>BV1tew5zVEDf</x:v>
       </x:c>
-      <x:c r="U227" s="17" t="str"/>
-      <x:c r="V227" s="27"/>
-      <x:c r="W227" s="17" t="str"/>
+      <x:c r="U227" s="17" t="str">
+        <x:v>张小珺商业访谈录</x:v>
+      </x:c>
+      <x:c r="V227" s="27" t="n">
+        <x:v>20260316</x:v>
+      </x:c>
+      <x:c r="W227" s="17" t="str">
+        <x:v>zhang-xiaojun-business-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="228" ht="42" customHeight="1">
       <x:c r="A228" s="22" t="str">
@@ -16794,9 +17178,15 @@
       <x:c r="T228" s="16" t="str">
         <x:v>BV1n2gD6gEoo</x:v>
       </x:c>
-      <x:c r="U228" s="17" t="str"/>
-      <x:c r="V228" s="27"/>
-      <x:c r="W228" s="17" t="str"/>
+      <x:c r="U228" s="17" t="str">
+        <x:v>卫诗婕｜漫谈播客集</x:v>
+      </x:c>
+      <x:c r="V228" s="27" t="n">
+        <x:v>20260723</x:v>
+      </x:c>
+      <x:c r="W228" s="17" t="str">
+        <x:v>wei-shijie-mantan-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="229" ht="42" customHeight="1">
       <x:c r="A229" s="22" t="str">
@@ -17314,9 +17704,15 @@
       <x:c r="T236" s="16" t="str">
         <x:v>BV1iVoVBgERD</x:v>
       </x:c>
-      <x:c r="U236" s="17" t="str"/>
-      <x:c r="V236" s="27"/>
-      <x:c r="W236" s="17" t="str"/>
+      <x:c r="U236" s="17" t="str">
+        <x:v>张小珺商业访谈录</x:v>
+      </x:c>
+      <x:c r="V236" s="27" t="n">
+        <x:v>20260424</x:v>
+      </x:c>
+      <x:c r="W236" s="17" t="str">
+        <x:v>zhang-xiaojun-business-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="237" ht="42" customHeight="1">
       <x:c r="A237" s="22" t="str">
@@ -17379,9 +17775,15 @@
       <x:c r="T237" s="16" t="str">
         <x:v>BV1N7oBYNEoU</x:v>
       </x:c>
-      <x:c r="U237" s="17" t="str"/>
-      <x:c r="V237" s="27"/>
-      <x:c r="W237" s="17" t="str"/>
+      <x:c r="U237" s="17" t="str">
+        <x:v>张小珺商业访谈录</x:v>
+      </x:c>
+      <x:c r="V237" s="27" t="n">
+        <x:v>20250323</x:v>
+      </x:c>
+      <x:c r="W237" s="17" t="str">
+        <x:v>zhang-xiaojun-business-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="238" ht="42" customHeight="1">
       <x:c r="A238" s="22" t="str">
@@ -17444,9 +17846,15 @@
       <x:c r="T238" s="16" t="str">
         <x:v>BV1VGjh6WEf9</x:v>
       </x:c>
-      <x:c r="U238" s="17" t="str"/>
-      <x:c r="V238" s="27"/>
-      <x:c r="W238" s="17" t="str"/>
+      <x:c r="U238" s="17" t="str">
+        <x:v>十字路口｜视频播客</x:v>
+      </x:c>
+      <x:c r="V238" s="27" t="n">
+        <x:v>20260621</x:v>
+      </x:c>
+      <x:c r="W238" s="17" t="str">
+        <x:v>crossroads-video-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="239" ht="42" customHeight="1">
       <x:c r="A239" s="22" t="str">
@@ -17574,9 +17982,15 @@
       <x:c r="T240" s="16" t="str">
         <x:v>BV12Lu16wEgL</x:v>
       </x:c>
-      <x:c r="U240" s="17" t="str"/>
-      <x:c r="V240" s="27"/>
-      <x:c r="W240" s="17" t="str"/>
+      <x:c r="U240" s="17" t="str">
+        <x:v>十字路口｜视频播客</x:v>
+      </x:c>
+      <x:c r="V240" s="27" t="n">
+        <x:v>20260809</x:v>
+      </x:c>
+      <x:c r="W240" s="17" t="str">
+        <x:v>crossroads-video-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="241" ht="42" customHeight="1">
       <x:c r="A241" s="22" t="str">
@@ -18419,9 +18833,15 @@
       <x:c r="T253" s="16" t="str">
         <x:v>BV12bNB6vEtt</x:v>
       </x:c>
-      <x:c r="U253" s="17" t="str"/>
-      <x:c r="V253" s="27"/>
-      <x:c r="W253" s="17" t="str"/>
+      <x:c r="U253" s="17" t="str">
+        <x:v>张小珺商业访谈录</x:v>
+      </x:c>
+      <x:c r="V253" s="27" t="n">
+        <x:v>20260716</x:v>
+      </x:c>
+      <x:c r="W253" s="17" t="str">
+        <x:v>zhang-xiaojun-business-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="254" ht="42" customHeight="1">
       <x:c r="A254" s="22" t="str">
@@ -18484,9 +18904,15 @@
       <x:c r="T254" s="16" t="str">
         <x:v>BV1ijuc6XEec</x:v>
       </x:c>
-      <x:c r="U254" s="17" t="str"/>
-      <x:c r="V254" s="27"/>
-      <x:c r="W254" s="17" t="str"/>
+      <x:c r="U254" s="17" t="str">
+        <x:v>卫诗婕｜漫谈播客集</x:v>
+      </x:c>
+      <x:c r="V254" s="27" t="n">
+        <x:v>20260804</x:v>
+      </x:c>
+      <x:c r="W254" s="17" t="str">
+        <x:v>wei-shijie-mantan-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="255" ht="42" customHeight="1">
       <x:c r="A255" s="22" t="str">
@@ -22591,9 +23017,15 @@
       <x:c r="T317" s="16" t="str">
         <x:v>YFjfBk8HI5o</x:v>
       </x:c>
-      <x:c r="U317" s="17" t="str"/>
-      <x:c r="V317" s="27"/>
-      <x:c r="W317" s="17" t="str"/>
+      <x:c r="U317" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V317" s="27" t="n">
+        <x:v>20260212</x:v>
+      </x:c>
+      <x:c r="W317" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="318" ht="42" customHeight="1">
       <x:c r="A318" s="22" t="str">
@@ -22656,9 +23088,15 @@
       <x:c r="T318" s="16" t="str">
         <x:v>EV7WhVT270Q</x:v>
       </x:c>
-      <x:c r="U318" s="17" t="str"/>
-      <x:c r="V318" s="27"/>
-      <x:c r="W318" s="17" t="str"/>
+      <x:c r="U318" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V318" s="27" t="n">
+        <x:v>20260131</x:v>
+      </x:c>
+      <x:c r="W318" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="319" ht="42" customHeight="1">
       <x:c r="A319" s="22" t="str">
@@ -22851,9 +23289,15 @@
       <x:c r="T321" s="16" t="str">
         <x:v>FUS6ceIvUnI</x:v>
       </x:c>
-      <x:c r="U321" s="17" t="str"/>
-      <x:c r="V321" s="27"/>
-      <x:c r="W321" s="17" t="str"/>
+      <x:c r="U321" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V321" s="27" t="n">
+        <x:v>20210731</x:v>
+      </x:c>
+      <x:c r="W321" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="322" ht="42" customHeight="1">
       <x:c r="A322" s="22" t="str">
@@ -22916,9 +23360,15 @@
       <x:c r="T322" s="16" t="str">
         <x:v>LRYkH-fAVGE</x:v>
       </x:c>
-      <x:c r="U322" s="17" t="str"/>
-      <x:c r="V322" s="27"/>
-      <x:c r="W322" s="17" t="str"/>
+      <x:c r="U322" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V322" s="27" t="n">
+        <x:v>20200721</x:v>
+      </x:c>
+      <x:c r="W322" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="323" ht="42" customHeight="1">
       <x:c r="A323" s="22" t="str">
@@ -23306,9 +23756,15 @@
       <x:c r="T328" s="16" t="str">
         <x:v>5jNsSC7ItWA</x:v>
       </x:c>
-      <x:c r="U328" s="17" t="str"/>
-      <x:c r="V328" s="27"/>
-      <x:c r="W328" s="17" t="str"/>
+      <x:c r="U328" s="17" t="str">
+        <x:v>Robot Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V328" s="27" t="n">
+        <x:v>20260227</x:v>
+      </x:c>
+      <x:c r="W328" s="17" t="str">
+        <x:v>robot-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="329" ht="42" customHeight="1">
       <x:c r="A329" s="22" t="str">
@@ -23371,9 +23827,15 @@
       <x:c r="T329" s="16" t="str">
         <x:v>0U1ayWbOkes</x:v>
       </x:c>
-      <x:c r="U329" s="17" t="str"/>
-      <x:c r="V329" s="27"/>
-      <x:c r="W329" s="17" t="str"/>
+      <x:c r="U329" s="17" t="str">
+        <x:v>Robot Talk Interviews</x:v>
+      </x:c>
+      <x:c r="V329" s="27" t="n">
+        <x:v>20240315</x:v>
+      </x:c>
+      <x:c r="W329" s="17" t="str">
+        <x:v>robot-talk-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="330" ht="42" customHeight="1">
       <x:c r="A330" s="22" t="str">
@@ -26202,9 +26664,15 @@
       <x:c r="T372" s="16" t="str">
         <x:v>A22Ej6kb2wo</x:v>
       </x:c>
-      <x:c r="U372" s="17" t="str"/>
-      <x:c r="V372" s="27"/>
-      <x:c r="W372" s="17" t="str"/>
+      <x:c r="U372" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V372" s="27" t="n">
+        <x:v>20200809</x:v>
+      </x:c>
+      <x:c r="W372" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="373" ht="42" customHeight="1">
       <x:c r="A373" s="22" t="str">
@@ -26267,9 +26735,15 @@
       <x:c r="T373" s="16" t="str">
         <x:v>kxi-_TT_-Nc</x:v>
       </x:c>
-      <x:c r="U373" s="17" t="str"/>
-      <x:c r="V373" s="27"/>
-      <x:c r="W373" s="17" t="str"/>
+      <x:c r="U373" s="17" t="str">
+        <x:v>Lex Fridman Podcast</x:v>
+      </x:c>
+      <x:c r="V373" s="27" t="n">
+        <x:v>20200714</x:v>
+      </x:c>
+      <x:c r="W373" s="17" t="str">
+        <x:v>lex-fridman-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="374" ht="42" customHeight="1">
       <x:c r="A374" s="22" t="str">
@@ -34665,9 +35139,15 @@
       <x:c r="T501" s="16" t="str">
         <x:v>48pxVdmkMIE</x:v>
       </x:c>
-      <x:c r="U501" s="17" t="str"/>
-      <x:c r="V501" s="27"/>
-      <x:c r="W501" s="17" t="str"/>
+      <x:c r="U501" s="17" t="str">
+        <x:v>Dwarkesh Patel Interviews</x:v>
+      </x:c>
+      <x:c r="V501" s="27" t="n">
+        <x:v>20250912</x:v>
+      </x:c>
+      <x:c r="W501" s="17" t="str">
+        <x:v>dwarkesh-patel-interviews</x:v>
+      </x:c>
     </x:row>
     <x:row r="502" ht="42" customHeight="1">
       <x:c r="A502" s="22" t="str">
@@ -35445,9 +35925,15 @@
       <x:c r="T513" s="16" t="str">
         <x:v>BV1KpCFBSEc6</x:v>
       </x:c>
-      <x:c r="U513" s="17" t="str"/>
-      <x:c r="V513" s="27"/>
-      <x:c r="W513" s="17" t="str"/>
+      <x:c r="U513" s="17" t="str">
+        <x:v>硅谷101｜AI Conversations</x:v>
+      </x:c>
+      <x:c r="V513" s="27" t="n">
+        <x:v>20251110</x:v>
+      </x:c>
+      <x:c r="W513" s="17" t="str">
+        <x:v>silicon-valley-101-ai-conversations</x:v>
+      </x:c>
     </x:row>
     <x:row r="514" ht="42" customHeight="1">
       <x:c r="A514" s="22" t="str">
@@ -35640,9 +36126,15 @@
       <x:c r="T516" s="16" t="str">
         <x:v>BV1ZGSoB5ETo</x:v>
       </x:c>
-      <x:c r="U516" s="17" t="str"/>
-      <x:c r="V516" s="27"/>
-      <x:c r="W516" s="17" t="str"/>
+      <x:c r="U516" s="17" t="str">
+        <x:v>卫诗婕｜漫谈播客集</x:v>
+      </x:c>
+      <x:c r="V516" s="27" t="n">
+        <x:v>20260406</x:v>
+      </x:c>
+      <x:c r="W516" s="17" t="str">
+        <x:v>wei-shijie-mantan-podcast</x:v>
+      </x:c>
     </x:row>
     <x:row r="517" ht="42" customHeight="1">
       <x:c r="A517" s="22" t="str">
@@ -37699,7 +38191,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eaad1485ebe4f0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8bbf136b5cc4c97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38021,7 +38513,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R824c6a55818a4bee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bbd0bca8b304f05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39023,7 +39515,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00bd5db7b35d41eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R098e87c724dd4d63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39222,16 +39714,16 @@
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="137" t="str">
-        <x:v>Course Series</x:v>
+        <x:v>Series Relationship</x:v>
       </x:c>
       <x:c r="B15" s="138" t="str">
-        <x:v>Stable Series ID, display title, and sequence order for related course videos</x:v>
+        <x:v>Stable Series ID, display title, and sequence order for related course lectures or interview episodes</x:v>
       </x:c>
       <x:c r="C15" s="138" t="str">
-        <x:v>Groups multiple lectures into one Course entry</x:v>
+        <x:v>Groups related videos into one Course or Interview entry</x:v>
       </x:c>
       <x:c r="D15" s="139" t="str">
-        <x:v>Apply only to confirmed course relationships; keep every canonical video as its own row.</x:v>
+        <x:v>Apply only to confirmed series relationships; keep every canonical video as its own row.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
@@ -39273,7 +39765,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B20" s="135" t="str">
-        <x:v>Multiple lectures from the same course are allowed; titles, links, and video IDs must remain unique.</x:v>
+        <x:v>Related course lectures or interview episodes may share a confirmed series; titles, links, and video IDs must remain unique.</x:v>
       </x:c>
       <x:c r="C20" s="135" t="str"/>
       <x:c r="D20" s="136" t="str"/>

</xml_diff>